<commit_message>
state: bot run 2026-09-16T05:01 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K981"/>
+  <dimension ref="A1:K1081"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42124,6 +42124,4252 @@
       <c r="K981" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 101.69 &lt;= EMA21 103.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D982" t="n">
+        <v>331.34</v>
+      </c>
+      <c r="E982" t="n">
+        <v>335.25</v>
+      </c>
+      <c r="F982" t="n">
+        <v>335.25</v>
+      </c>
+      <c r="G982" t="n">
+        <v>325.97</v>
+      </c>
+      <c r="H982" t="n">
+        <v>321.13</v>
+      </c>
+      <c r="I982" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J982" t="b">
+        <v>0</v>
+      </c>
+      <c r="K982" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 331.34 &lt;= Upper 335.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D983" t="n">
+        <v>497.12</v>
+      </c>
+      <c r="E983" t="n">
+        <v>514.87</v>
+      </c>
+      <c r="F983" t="n">
+        <v>514.87</v>
+      </c>
+      <c r="G983" t="n">
+        <v>498</v>
+      </c>
+      <c r="H983" t="n">
+        <v>492.09</v>
+      </c>
+      <c r="I983" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J983" t="b">
+        <v>0</v>
+      </c>
+      <c r="K983" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 497.12 &lt;= Upper 514.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D984" t="n">
+        <v>212.17</v>
+      </c>
+      <c r="E984" t="n">
+        <v>231.3</v>
+      </c>
+      <c r="F984" t="n">
+        <v>231.3</v>
+      </c>
+      <c r="G984" t="n">
+        <v>217.93</v>
+      </c>
+      <c r="H984" t="n">
+        <v>218.14</v>
+      </c>
+      <c r="I984" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J984" t="b">
+        <v>0</v>
+      </c>
+      <c r="K984" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 217.93 &lt;= EMA21 218.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D985" t="n">
+        <v>344.98</v>
+      </c>
+      <c r="E985" t="n">
+        <v>351.26</v>
+      </c>
+      <c r="F985" t="n">
+        <v>351.26</v>
+      </c>
+      <c r="G985" t="n">
+        <v>340.83</v>
+      </c>
+      <c r="H985" t="n">
+        <v>341.85</v>
+      </c>
+      <c r="I985" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J985" t="b">
+        <v>0</v>
+      </c>
+      <c r="K985" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 340.83 &lt;= EMA21 341.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D986" t="n">
+        <v>341.43</v>
+      </c>
+      <c r="E986" t="n">
+        <v>347.54</v>
+      </c>
+      <c r="F986" t="n">
+        <v>347.54</v>
+      </c>
+      <c r="G986" t="n">
+        <v>337.68</v>
+      </c>
+      <c r="H986" t="n">
+        <v>338.96</v>
+      </c>
+      <c r="I986" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J986" t="b">
+        <v>0</v>
+      </c>
+      <c r="K986" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 337.68 &lt;= EMA21 338.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D987" t="n">
+        <v>248.42</v>
+      </c>
+      <c r="E987" t="n">
+        <v>266.79</v>
+      </c>
+      <c r="F987" t="n">
+        <v>266.79</v>
+      </c>
+      <c r="G987" t="n">
+        <v>254.31</v>
+      </c>
+      <c r="H987" t="n">
+        <v>256.71</v>
+      </c>
+      <c r="I987" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J987" t="b">
+        <v>0</v>
+      </c>
+      <c r="K987" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 254.31 &lt;= EMA21 256.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D988" t="n">
+        <v>670.24</v>
+      </c>
+      <c r="E988" t="n">
+        <v>679.6799999999999</v>
+      </c>
+      <c r="F988" t="n">
+        <v>679.6799999999999</v>
+      </c>
+      <c r="G988" t="n">
+        <v>637.8</v>
+      </c>
+      <c r="H988" t="n">
+        <v>613.29</v>
+      </c>
+      <c r="I988" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J988" t="b">
+        <v>0</v>
+      </c>
+      <c r="K988" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 670.24 &lt;= Upper 679.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D989" t="n">
+        <v>356.58</v>
+      </c>
+      <c r="E989" t="n">
+        <v>376.22</v>
+      </c>
+      <c r="F989" t="n">
+        <v>376.22</v>
+      </c>
+      <c r="G989" t="n">
+        <v>360.69</v>
+      </c>
+      <c r="H989" t="n">
+        <v>356.5</v>
+      </c>
+      <c r="I989" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J989" t="b">
+        <v>0</v>
+      </c>
+      <c r="K989" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 356.58 &lt;= Upper 376.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D990" t="n">
+        <v>339.27</v>
+      </c>
+      <c r="E990" t="n">
+        <v>381.03</v>
+      </c>
+      <c r="F990" t="n">
+        <v>381.03</v>
+      </c>
+      <c r="G990" t="n">
+        <v>356.05</v>
+      </c>
+      <c r="H990" t="n">
+        <v>365.79</v>
+      </c>
+      <c r="I990" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J990" t="b">
+        <v>0</v>
+      </c>
+      <c r="K990" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 356.05 &lt;= EMA21 365.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D991" t="n">
+        <v>140.35</v>
+      </c>
+      <c r="E991" t="n">
+        <v>162.03</v>
+      </c>
+      <c r="F991" t="n">
+        <v>162.03</v>
+      </c>
+      <c r="G991" t="n">
+        <v>149.38</v>
+      </c>
+      <c r="H991" t="n">
+        <v>148.72</v>
+      </c>
+      <c r="I991" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J991" t="b">
+        <v>0</v>
+      </c>
+      <c r="K991" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 140.35 &lt;= Upper 162.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D992" t="n">
+        <v>255.65</v>
+      </c>
+      <c r="E992" t="n">
+        <v>286.11</v>
+      </c>
+      <c r="F992" t="n">
+        <v>286.11</v>
+      </c>
+      <c r="G992" t="n">
+        <v>250.36</v>
+      </c>
+      <c r="H992" t="n">
+        <v>236.78</v>
+      </c>
+      <c r="I992" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J992" t="b">
+        <v>0</v>
+      </c>
+      <c r="K992" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 255.65 &lt;= Upper 286.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D993" t="n">
+        <v>257.76</v>
+      </c>
+      <c r="E993" t="n">
+        <v>298.42</v>
+      </c>
+      <c r="F993" t="n">
+        <v>298.42</v>
+      </c>
+      <c r="G993" t="n">
+        <v>262.72</v>
+      </c>
+      <c r="H993" t="n">
+        <v>265.42</v>
+      </c>
+      <c r="I993" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J993" t="b">
+        <v>0</v>
+      </c>
+      <c r="K993" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 262.72 &lt;= EMA21 265.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D994" t="n">
+        <v>504.2</v>
+      </c>
+      <c r="E994" t="n">
+        <v>521.13</v>
+      </c>
+      <c r="F994" t="n">
+        <v>521.13</v>
+      </c>
+      <c r="G994" t="n">
+        <v>496.01</v>
+      </c>
+      <c r="H994" t="n">
+        <v>489.1</v>
+      </c>
+      <c r="I994" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J994" t="b">
+        <v>0</v>
+      </c>
+      <c r="K994" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 504.20 &lt;= Upper 521.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D995" t="n">
+        <v>97.14</v>
+      </c>
+      <c r="E995" t="n">
+        <v>105.65</v>
+      </c>
+      <c r="F995" t="n">
+        <v>105.65</v>
+      </c>
+      <c r="G995" t="n">
+        <v>98.03</v>
+      </c>
+      <c r="H995" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="I995" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J995" t="b">
+        <v>0</v>
+      </c>
+      <c r="K995" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 97.14 &lt;= Upper 105.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D996" t="n">
+        <v>927.6</v>
+      </c>
+      <c r="E996" t="n">
+        <v>1019.26</v>
+      </c>
+      <c r="F996" t="n">
+        <v>1019.26</v>
+      </c>
+      <c r="G996" t="n">
+        <v>959.6900000000001</v>
+      </c>
+      <c r="H996" t="n">
+        <v>953.62</v>
+      </c>
+      <c r="I996" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J996" t="b">
+        <v>0</v>
+      </c>
+      <c r="K996" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 927.60 &lt;= Upper 1019.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D997" t="n">
+        <v>187.8</v>
+      </c>
+      <c r="E997" t="n">
+        <v>185.65</v>
+      </c>
+      <c r="F997" t="n">
+        <v>185.65</v>
+      </c>
+      <c r="G997" t="n">
+        <v>177.22</v>
+      </c>
+      <c r="H997" t="n">
+        <v>171.59</v>
+      </c>
+      <c r="I997" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J997" t="b">
+        <v>0</v>
+      </c>
+      <c r="K997" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.18x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="D998" t="n">
+        <v>263.43</v>
+      </c>
+      <c r="E998" t="n">
+        <v>271.55</v>
+      </c>
+      <c r="F998" t="n">
+        <v>271.55</v>
+      </c>
+      <c r="G998" t="n">
+        <v>262.03</v>
+      </c>
+      <c r="H998" t="n">
+        <v>264.27</v>
+      </c>
+      <c r="I998" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J998" t="b">
+        <v>0</v>
+      </c>
+      <c r="K998" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 262.03 &lt;= EMA21 264.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D999" t="n">
+        <v>421.17</v>
+      </c>
+      <c r="E999" t="n">
+        <v>516.41</v>
+      </c>
+      <c r="F999" t="n">
+        <v>516.41</v>
+      </c>
+      <c r="G999" t="n">
+        <v>446.78</v>
+      </c>
+      <c r="H999" t="n">
+        <v>466.69</v>
+      </c>
+      <c r="I999" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J999" t="b">
+        <v>0</v>
+      </c>
+      <c r="K999" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 446.78 &lt;= EMA21 466.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D1000" t="n">
+        <v>270.87</v>
+      </c>
+      <c r="E1000" t="n">
+        <v>333.71</v>
+      </c>
+      <c r="F1000" t="n">
+        <v>333.71</v>
+      </c>
+      <c r="G1000" t="n">
+        <v>292.74</v>
+      </c>
+      <c r="H1000" t="n">
+        <v>301.6</v>
+      </c>
+      <c r="I1000" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1000" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1000" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 292.74 &lt;= EMA21 301.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D1001" t="n">
+        <v>168.02</v>
+      </c>
+      <c r="E1001" t="n">
+        <v>194.62</v>
+      </c>
+      <c r="F1001" t="n">
+        <v>194.62</v>
+      </c>
+      <c r="G1001" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="H1001" t="n">
+        <v>181.84</v>
+      </c>
+      <c r="I1001" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1001" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1001" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 176.30 &lt;= EMA21 181.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D1002" t="n">
+        <v>1591.48</v>
+      </c>
+      <c r="E1002" t="n">
+        <v>1823.66</v>
+      </c>
+      <c r="F1002" t="n">
+        <v>1823.66</v>
+      </c>
+      <c r="G1002" t="n">
+        <v>1664.18</v>
+      </c>
+      <c r="H1002" t="n">
+        <v>1698.05</v>
+      </c>
+      <c r="I1002" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="J1002" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1002" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1664.18 &lt;= EMA21 1698.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D1003" t="n">
+        <v>361.35</v>
+      </c>
+      <c r="E1003" t="n">
+        <v>379.93</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>379.93</v>
+      </c>
+      <c r="G1003" t="n">
+        <v>364.25</v>
+      </c>
+      <c r="H1003" t="n">
+        <v>366.93</v>
+      </c>
+      <c r="I1003" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J1003" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1003" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 364.25 &lt;= EMA21 366.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D1004" t="n">
+        <v>221.7</v>
+      </c>
+      <c r="E1004" t="n">
+        <v>253.12</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>253.12</v>
+      </c>
+      <c r="G1004" t="n">
+        <v>224.35</v>
+      </c>
+      <c r="H1004" t="n">
+        <v>223.48</v>
+      </c>
+      <c r="I1004" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J1004" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1004" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 221.70 &lt;= Upper 253.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="D1005" t="n">
+        <v>226.35</v>
+      </c>
+      <c r="E1005" t="n">
+        <v>232.01</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>232.01</v>
+      </c>
+      <c r="G1005" t="n">
+        <v>226.84</v>
+      </c>
+      <c r="H1005" t="n">
+        <v>229</v>
+      </c>
+      <c r="I1005" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1005" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1005" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 226.84 &lt;= EMA21 229.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D1006" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="E1006" t="n">
+        <v>77.86</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>77.86</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="H1006" t="n">
+        <v>74.73999999999999</v>
+      </c>
+      <c r="I1006" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J1006" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1006" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 72.90 &lt;= EMA21 74.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D1007" t="n">
+        <v>1142.46</v>
+      </c>
+      <c r="E1007" t="n">
+        <v>1364.77</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>1364.77</v>
+      </c>
+      <c r="G1007" t="n">
+        <v>1197.76</v>
+      </c>
+      <c r="H1007" t="n">
+        <v>1245.1</v>
+      </c>
+      <c r="I1007" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1007" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1007" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1197.76 &lt;= EMA21 1245.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D1008" t="n">
+        <v>90</v>
+      </c>
+      <c r="E1008" t="n">
+        <v>87.62</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>87.62</v>
+      </c>
+      <c r="G1008" t="n">
+        <v>80.08</v>
+      </c>
+      <c r="H1008" t="n">
+        <v>74.59</v>
+      </c>
+      <c r="I1008" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="J1008" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1008" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D1009" t="n">
+        <v>118.06</v>
+      </c>
+      <c r="E1009" t="n">
+        <v>115.98</v>
+      </c>
+      <c r="F1009" t="n">
+        <v>115.98</v>
+      </c>
+      <c r="G1009" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="H1009" t="n">
+        <v>103.07</v>
+      </c>
+      <c r="I1009" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J1009" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1009" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D1010" t="n">
+        <v>332.85</v>
+      </c>
+      <c r="E1010" t="n">
+        <v>402.68</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>402.68</v>
+      </c>
+      <c r="G1010" t="n">
+        <v>354.45</v>
+      </c>
+      <c r="H1010" t="n">
+        <v>362.03</v>
+      </c>
+      <c r="I1010" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1010" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1010" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 354.45 &lt;= EMA21 362.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>ENTG</t>
+        </is>
+      </c>
+      <c r="D1011" t="n">
+        <v>129.64</v>
+      </c>
+      <c r="E1011" t="n">
+        <v>150.77</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>150.77</v>
+      </c>
+      <c r="G1011" t="n">
+        <v>135.3</v>
+      </c>
+      <c r="H1011" t="n">
+        <v>138.05</v>
+      </c>
+      <c r="I1011" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1011" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1011" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.30 &lt;= EMA21 138.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+      <c r="D1012" t="n">
+        <v>71.48999999999999</v>
+      </c>
+      <c r="E1012" t="n">
+        <v>77.25</v>
+      </c>
+      <c r="F1012" t="n">
+        <v>77.25</v>
+      </c>
+      <c r="G1012" t="n">
+        <v>72.69</v>
+      </c>
+      <c r="H1012" t="n">
+        <v>74.11</v>
+      </c>
+      <c r="I1012" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J1012" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1012" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 72.69 &lt;= EMA21 74.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D1013" t="n">
+        <v>35.64</v>
+      </c>
+      <c r="E1013" t="n">
+        <v>40.31</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>40.31</v>
+      </c>
+      <c r="G1013" t="n">
+        <v>37.67</v>
+      </c>
+      <c r="H1013" t="n">
+        <v>36.96</v>
+      </c>
+      <c r="I1013" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J1013" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1013" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 35.64 &lt;= Upper 40.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D1014" t="n">
+        <v>543.51</v>
+      </c>
+      <c r="E1014" t="n">
+        <v>573.16</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>573.16</v>
+      </c>
+      <c r="G1014" t="n">
+        <v>523.59</v>
+      </c>
+      <c r="H1014" t="n">
+        <v>496.26</v>
+      </c>
+      <c r="I1014" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J1014" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1014" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 543.51 &lt;= Upper 573.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D1015" t="n">
+        <v>33.82</v>
+      </c>
+      <c r="E1015" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="G1015" t="n">
+        <v>32.87</v>
+      </c>
+      <c r="H1015" t="n">
+        <v>31.34</v>
+      </c>
+      <c r="I1015" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J1015" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1015" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 33.82 &lt;= Upper 34.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="D1016" t="n">
+        <v>411.96</v>
+      </c>
+      <c r="E1016" t="n">
+        <v>494.62</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>494.62</v>
+      </c>
+      <c r="G1016" t="n">
+        <v>445.64</v>
+      </c>
+      <c r="H1016" t="n">
+        <v>459.11</v>
+      </c>
+      <c r="I1016" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J1016" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1016" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 445.64 &lt;= EMA21 459.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D1017" t="n">
+        <v>771.8099999999999</v>
+      </c>
+      <c r="E1017" t="n">
+        <v>906.27</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>906.27</v>
+      </c>
+      <c r="G1017" t="n">
+        <v>827.15</v>
+      </c>
+      <c r="H1017" t="n">
+        <v>838.89</v>
+      </c>
+      <c r="I1017" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1017" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1017" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 827.15 &lt;= EMA21 838.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="D1018" t="n">
+        <v>192.84</v>
+      </c>
+      <c r="E1018" t="n">
+        <v>202.21</v>
+      </c>
+      <c r="F1018" t="n">
+        <v>202.21</v>
+      </c>
+      <c r="G1018" t="n">
+        <v>192.55</v>
+      </c>
+      <c r="H1018" t="n">
+        <v>191.88</v>
+      </c>
+      <c r="I1018" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1018" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1018" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 192.84 &lt;= Upper 202.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D1019" t="n">
+        <v>110.07</v>
+      </c>
+      <c r="E1019" t="n">
+        <v>112.73</v>
+      </c>
+      <c r="F1019" t="n">
+        <v>112.73</v>
+      </c>
+      <c r="G1019" t="n">
+        <v>109.97</v>
+      </c>
+      <c r="H1019" t="n">
+        <v>111</v>
+      </c>
+      <c r="I1019" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J1019" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1019" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 109.97 &lt;= EMA21 111.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="D1020" t="n">
+        <v>193.4</v>
+      </c>
+      <c r="E1020" t="n">
+        <v>197.02</v>
+      </c>
+      <c r="F1020" t="n">
+        <v>197.02</v>
+      </c>
+      <c r="G1020" t="n">
+        <v>186.89</v>
+      </c>
+      <c r="H1020" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="I1020" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J1020" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 193.40 &lt;= Upper 197.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="D1021" t="n">
+        <v>248.37</v>
+      </c>
+      <c r="E1021" t="n">
+        <v>246.87</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>246.87</v>
+      </c>
+      <c r="G1021" t="n">
+        <v>240.8</v>
+      </c>
+      <c r="H1021" t="n">
+        <v>237.41</v>
+      </c>
+      <c r="I1021" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J1021" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1021" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.89x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D1022" t="n">
+        <v>141.9</v>
+      </c>
+      <c r="E1022" t="n">
+        <v>150.71</v>
+      </c>
+      <c r="F1022" t="n">
+        <v>150.71</v>
+      </c>
+      <c r="G1022" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="H1022" t="n">
+        <v>133.65</v>
+      </c>
+      <c r="I1022" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1022" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1022" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 141.90 &lt;= Upper 150.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D1023" t="n">
+        <v>329.27</v>
+      </c>
+      <c r="E1023" t="n">
+        <v>379.33</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>379.33</v>
+      </c>
+      <c r="G1023" t="n">
+        <v>330.66</v>
+      </c>
+      <c r="H1023" t="n">
+        <v>334.51</v>
+      </c>
+      <c r="I1023" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J1023" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1023" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 330.66 &lt;= EMA21 334.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D1024" t="n">
+        <v>375.09</v>
+      </c>
+      <c r="E1024" t="n">
+        <v>390.27</v>
+      </c>
+      <c r="F1024" t="n">
+        <v>390.27</v>
+      </c>
+      <c r="G1024" t="n">
+        <v>352.84</v>
+      </c>
+      <c r="H1024" t="n">
+        <v>352.52</v>
+      </c>
+      <c r="I1024" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1024" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 375.09 &lt;= Upper 390.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D1025" t="n">
+        <v>242.49</v>
+      </c>
+      <c r="E1025" t="n">
+        <v>241.84</v>
+      </c>
+      <c r="F1025" t="n">
+        <v>241.84</v>
+      </c>
+      <c r="G1025" t="n">
+        <v>220.24</v>
+      </c>
+      <c r="H1025" t="n">
+        <v>213.53</v>
+      </c>
+      <c r="I1025" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J1025" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1025" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D1026" t="n">
+        <v>322.98</v>
+      </c>
+      <c r="E1026" t="n">
+        <v>347.77</v>
+      </c>
+      <c r="F1026" t="n">
+        <v>347.77</v>
+      </c>
+      <c r="G1026" t="n">
+        <v>329.25</v>
+      </c>
+      <c r="H1026" t="n">
+        <v>325.59</v>
+      </c>
+      <c r="I1026" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J1026" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1026" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 322.98 &lt;= Upper 347.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D1027" t="n">
+        <v>172.56</v>
+      </c>
+      <c r="E1027" t="n">
+        <v>187.98</v>
+      </c>
+      <c r="F1027" t="n">
+        <v>187.98</v>
+      </c>
+      <c r="G1027" t="n">
+        <v>172.31</v>
+      </c>
+      <c r="H1027" t="n">
+        <v>171.11</v>
+      </c>
+      <c r="I1027" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1027" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1027" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 172.56 &lt;= Upper 187.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D1028" t="n">
+        <v>230.27</v>
+      </c>
+      <c r="E1028" t="n">
+        <v>247.65</v>
+      </c>
+      <c r="F1028" t="n">
+        <v>247.65</v>
+      </c>
+      <c r="G1028" t="n">
+        <v>224.7</v>
+      </c>
+      <c r="H1028" t="n">
+        <v>229.22</v>
+      </c>
+      <c r="I1028" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J1028" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1028" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 224.70 &lt;= EMA21 229.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D1029" t="n">
+        <v>193.89</v>
+      </c>
+      <c r="E1029" t="n">
+        <v>196.71</v>
+      </c>
+      <c r="F1029" t="n">
+        <v>196.71</v>
+      </c>
+      <c r="G1029" t="n">
+        <v>177.84</v>
+      </c>
+      <c r="H1029" t="n">
+        <v>174.99</v>
+      </c>
+      <c r="I1029" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J1029" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1029" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 193.89 &lt;= Upper 196.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D1030" t="n">
+        <v>327.23</v>
+      </c>
+      <c r="E1030" t="n">
+        <v>329.36</v>
+      </c>
+      <c r="F1030" t="n">
+        <v>329.36</v>
+      </c>
+      <c r="G1030" t="n">
+        <v>308.99</v>
+      </c>
+      <c r="H1030" t="n">
+        <v>300.02</v>
+      </c>
+      <c r="I1030" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1030" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1030" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 327.23 &lt;= Upper 329.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="D1031" t="n">
+        <v>377.67</v>
+      </c>
+      <c r="E1031" t="n">
+        <v>468.2</v>
+      </c>
+      <c r="F1031" t="n">
+        <v>468.2</v>
+      </c>
+      <c r="G1031" t="n">
+        <v>380.12</v>
+      </c>
+      <c r="H1031" t="n">
+        <v>390.1</v>
+      </c>
+      <c r="I1031" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J1031" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1031" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 380.12 &lt;= EMA21 390.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D1032" t="n">
+        <v>172.37</v>
+      </c>
+      <c r="E1032" t="n">
+        <v>173.63</v>
+      </c>
+      <c r="F1032" t="n">
+        <v>173.63</v>
+      </c>
+      <c r="G1032" t="n">
+        <v>162.88</v>
+      </c>
+      <c r="H1032" t="n">
+        <v>160.78</v>
+      </c>
+      <c r="I1032" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J1032" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1032" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 172.37 &lt;= Upper 173.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D1033" t="n">
+        <v>189.81</v>
+      </c>
+      <c r="E1033" t="n">
+        <v>200.24</v>
+      </c>
+      <c r="F1033" t="n">
+        <v>200.24</v>
+      </c>
+      <c r="G1033" t="n">
+        <v>184.76</v>
+      </c>
+      <c r="H1033" t="n">
+        <v>174.96</v>
+      </c>
+      <c r="I1033" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J1033" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1033" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 189.81 &lt;= Upper 200.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>WDAY</t>
+        </is>
+      </c>
+      <c r="D1034" t="n">
+        <v>190.67</v>
+      </c>
+      <c r="E1034" t="n">
+        <v>207.37</v>
+      </c>
+      <c r="F1034" t="n">
+        <v>207.37</v>
+      </c>
+      <c r="G1034" t="n">
+        <v>191.43</v>
+      </c>
+      <c r="H1034" t="n">
+        <v>189.9</v>
+      </c>
+      <c r="I1034" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J1034" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1034" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 190.67 &lt;= Upper 207.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="D1035" t="n">
+        <v>241.96</v>
+      </c>
+      <c r="E1035" t="n">
+        <v>264.99</v>
+      </c>
+      <c r="F1035" t="n">
+        <v>264.99</v>
+      </c>
+      <c r="G1035" t="n">
+        <v>240.04</v>
+      </c>
+      <c r="H1035" t="n">
+        <v>238.89</v>
+      </c>
+      <c r="I1035" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J1035" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1035" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 241.96 &lt;= Upper 264.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="D1036" t="n">
+        <v>266.62</v>
+      </c>
+      <c r="E1036" t="n">
+        <v>292.92</v>
+      </c>
+      <c r="F1036" t="n">
+        <v>292.92</v>
+      </c>
+      <c r="G1036" t="n">
+        <v>266.33</v>
+      </c>
+      <c r="H1036" t="n">
+        <v>259.35</v>
+      </c>
+      <c r="I1036" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J1036" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1036" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 266.62 &lt;= Upper 292.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D1037" t="n">
+        <v>93.06999999999999</v>
+      </c>
+      <c r="E1037" t="n">
+        <v>108.56</v>
+      </c>
+      <c r="F1037" t="n">
+        <v>108.56</v>
+      </c>
+      <c r="G1037" t="n">
+        <v>96.05</v>
+      </c>
+      <c r="H1037" t="n">
+        <v>97.77</v>
+      </c>
+      <c r="I1037" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1037" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1037" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 96.05 &lt;= EMA21 97.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D1038" t="n">
+        <v>190.45</v>
+      </c>
+      <c r="E1038" t="n">
+        <v>197.55</v>
+      </c>
+      <c r="F1038" t="n">
+        <v>197.55</v>
+      </c>
+      <c r="G1038" t="n">
+        <v>174.41</v>
+      </c>
+      <c r="H1038" t="n">
+        <v>164.05</v>
+      </c>
+      <c r="I1038" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J1038" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1038" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 190.45 &lt;= Upper 197.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="D1039" t="n">
+        <v>331.46</v>
+      </c>
+      <c r="E1039" t="n">
+        <v>331.25</v>
+      </c>
+      <c r="F1039" t="n">
+        <v>331.25</v>
+      </c>
+      <c r="G1039" t="n">
+        <v>321.56</v>
+      </c>
+      <c r="H1039" t="n">
+        <v>325.51</v>
+      </c>
+      <c r="I1039" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1039" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1039" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 321.56 &lt;= EMA21 325.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="D1040" t="n">
+        <v>442.08</v>
+      </c>
+      <c r="E1040" t="n">
+        <v>679.28</v>
+      </c>
+      <c r="F1040" t="n">
+        <v>679.28</v>
+      </c>
+      <c r="G1040" t="n">
+        <v>495.49</v>
+      </c>
+      <c r="H1040" t="n">
+        <v>530.1900000000001</v>
+      </c>
+      <c r="I1040" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J1040" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1040" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 495.49 &lt;= EMA21 530.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="D1041" t="n">
+        <v>273.96</v>
+      </c>
+      <c r="E1041" t="n">
+        <v>353.84</v>
+      </c>
+      <c r="F1041" t="n">
+        <v>353.84</v>
+      </c>
+      <c r="G1041" t="n">
+        <v>290.19</v>
+      </c>
+      <c r="H1041" t="n">
+        <v>305.49</v>
+      </c>
+      <c r="I1041" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J1041" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1041" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 290.19 &lt;= EMA21 305.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D1042" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="E1042" t="n">
+        <v>450.73</v>
+      </c>
+      <c r="F1042" t="n">
+        <v>450.73</v>
+      </c>
+      <c r="G1042" t="n">
+        <v>392.9</v>
+      </c>
+      <c r="H1042" t="n">
+        <v>402.14</v>
+      </c>
+      <c r="I1042" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J1042" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1042" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 392.90 &lt;= EMA21 402.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D1043" t="n">
+        <v>226.5</v>
+      </c>
+      <c r="E1043" t="n">
+        <v>278.36</v>
+      </c>
+      <c r="F1043" t="n">
+        <v>278.36</v>
+      </c>
+      <c r="G1043" t="n">
+        <v>225.34</v>
+      </c>
+      <c r="H1043" t="n">
+        <v>232.91</v>
+      </c>
+      <c r="I1043" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J1043" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 225.34 &lt;= EMA21 232.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="J1044" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1044" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D1045" t="n">
+        <v>132.75</v>
+      </c>
+      <c r="E1045" t="n">
+        <v>166.7</v>
+      </c>
+      <c r="F1045" t="n">
+        <v>166.7</v>
+      </c>
+      <c r="G1045" t="n">
+        <v>136.96</v>
+      </c>
+      <c r="H1045" t="n">
+        <v>141.29</v>
+      </c>
+      <c r="I1045" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J1045" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1045" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 136.96 &lt;= EMA21 141.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>TYL</t>
+        </is>
+      </c>
+      <c r="D1046" t="n">
+        <v>353.13</v>
+      </c>
+      <c r="E1046" t="n">
+        <v>385.91</v>
+      </c>
+      <c r="F1046" t="n">
+        <v>385.91</v>
+      </c>
+      <c r="G1046" t="n">
+        <v>352.61</v>
+      </c>
+      <c r="H1046" t="n">
+        <v>349.66</v>
+      </c>
+      <c r="I1046" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J1046" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1046" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 353.13 &lt;= Upper 385.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="D1047" t="n">
+        <v>147.22</v>
+      </c>
+      <c r="E1047" t="n">
+        <v>161.91</v>
+      </c>
+      <c r="F1047" t="n">
+        <v>161.91</v>
+      </c>
+      <c r="G1047" t="n">
+        <v>147.37</v>
+      </c>
+      <c r="H1047" t="n">
+        <v>147.91</v>
+      </c>
+      <c r="I1047" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1047" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1047" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 147.37 &lt;= EMA21 147.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1048" t="n">
+        <v>195.62</v>
+      </c>
+      <c r="E1048" t="n">
+        <v>209.3</v>
+      </c>
+      <c r="F1048" t="n">
+        <v>209.3</v>
+      </c>
+      <c r="G1048" t="n">
+        <v>186.56</v>
+      </c>
+      <c r="H1048" t="n">
+        <v>184.87</v>
+      </c>
+      <c r="I1048" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1048" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1048" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 195.62 &lt;= Upper 209.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D1049" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="E1049" t="n">
+        <v>66.26000000000001</v>
+      </c>
+      <c r="F1049" t="n">
+        <v>66.26000000000001</v>
+      </c>
+      <c r="G1049" t="n">
+        <v>61.77</v>
+      </c>
+      <c r="H1049" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="I1049" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1049" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1049" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 63.28 &lt;= Upper 66.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1050" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="E1050" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="F1050" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="G1050" t="n">
+        <v>11.41</v>
+      </c>
+      <c r="H1050" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="I1050" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J1050" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1050" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11.41 &lt;= EMA21 11.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D1051" t="n">
+        <v>123.51</v>
+      </c>
+      <c r="E1051" t="n">
+        <v>125.45</v>
+      </c>
+      <c r="F1051" t="n">
+        <v>125.45</v>
+      </c>
+      <c r="G1051" t="n">
+        <v>118.42</v>
+      </c>
+      <c r="H1051" t="n">
+        <v>113.79</v>
+      </c>
+      <c r="I1051" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J1051" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1051" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 123.51 &lt;= Upper 125.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>GEN</t>
+        </is>
+      </c>
+      <c r="D1052" t="n">
+        <v>31.23</v>
+      </c>
+      <c r="E1052" t="n">
+        <v>32.23</v>
+      </c>
+      <c r="F1052" t="n">
+        <v>32.23</v>
+      </c>
+      <c r="G1052" t="n">
+        <v>30.56</v>
+      </c>
+      <c r="H1052" t="n">
+        <v>29.91</v>
+      </c>
+      <c r="I1052" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1052" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1052" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 31.23 &lt;= Upper 32.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D1053" t="n">
+        <v>153.74</v>
+      </c>
+      <c r="E1053" t="n">
+        <v>159.76</v>
+      </c>
+      <c r="F1053" t="n">
+        <v>159.76</v>
+      </c>
+      <c r="G1053" t="n">
+        <v>149.32</v>
+      </c>
+      <c r="H1053" t="n">
+        <v>146.1</v>
+      </c>
+      <c r="I1053" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1053" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1053" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 153.74 &lt;= Upper 159.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D1054" t="n">
+        <v>430.88</v>
+      </c>
+      <c r="E1054" t="n">
+        <v>422.92</v>
+      </c>
+      <c r="F1054" t="n">
+        <v>422.92</v>
+      </c>
+      <c r="G1054" t="n">
+        <v>407.52</v>
+      </c>
+      <c r="H1054" t="n">
+        <v>402.25</v>
+      </c>
+      <c r="I1054" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J1054" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1054" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>JNPR</t>
+        </is>
+      </c>
+      <c r="J1055" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1055" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="D1056" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="E1056" t="n">
+        <v>113.73</v>
+      </c>
+      <c r="F1056" t="n">
+        <v>113.73</v>
+      </c>
+      <c r="G1056" t="n">
+        <v>106.79</v>
+      </c>
+      <c r="H1056" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="I1056" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J1056" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1056" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.79 &lt;= EMA21 109.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="J1057" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1057" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="D1058" t="n">
+        <v>211.91</v>
+      </c>
+      <c r="E1058" t="n">
+        <v>247.17</v>
+      </c>
+      <c r="F1058" t="n">
+        <v>247.17</v>
+      </c>
+      <c r="G1058" t="n">
+        <v>217.44</v>
+      </c>
+      <c r="H1058" t="n">
+        <v>223.75</v>
+      </c>
+      <c r="I1058" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1058" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1058" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 217.44 &lt;= EMA21 223.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D1059" t="n">
+        <v>50.24</v>
+      </c>
+      <c r="E1059" t="n">
+        <v>49.84</v>
+      </c>
+      <c r="F1059" t="n">
+        <v>49.84</v>
+      </c>
+      <c r="G1059" t="n">
+        <v>45.93</v>
+      </c>
+      <c r="H1059" t="n">
+        <v>43.41</v>
+      </c>
+      <c r="I1059" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1059" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1059" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.78x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D1060" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="E1060" t="n">
+        <v>47.82</v>
+      </c>
+      <c r="F1060" t="n">
+        <v>47.82</v>
+      </c>
+      <c r="G1060" t="n">
+        <v>42.92</v>
+      </c>
+      <c r="H1060" t="n">
+        <v>42.44</v>
+      </c>
+      <c r="I1060" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1060" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1060" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 43.01 &lt;= Upper 47.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D1061" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="E1061" t="n">
+        <v>83.89</v>
+      </c>
+      <c r="F1061" t="n">
+        <v>83.89</v>
+      </c>
+      <c r="G1061" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="H1061" t="n">
+        <v>78.45</v>
+      </c>
+      <c r="I1061" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J1061" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1061" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 77.90 &lt;= Upper 83.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D1062" t="n">
+        <v>106.42</v>
+      </c>
+      <c r="E1062" t="n">
+        <v>110.99</v>
+      </c>
+      <c r="F1062" t="n">
+        <v>110.99</v>
+      </c>
+      <c r="G1062" t="n">
+        <v>106.61</v>
+      </c>
+      <c r="H1062" t="n">
+        <v>106.03</v>
+      </c>
+      <c r="I1062" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J1062" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1062" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 106.42 &lt;= Upper 110.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="D1063" t="n">
+        <v>28.03</v>
+      </c>
+      <c r="E1063" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="F1063" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="G1063" t="n">
+        <v>28.16</v>
+      </c>
+      <c r="H1063" t="n">
+        <v>28.07</v>
+      </c>
+      <c r="I1063" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J1063" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1063" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 28.03 &lt;= Upper 28.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="D1064" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1064" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="F1064" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G1064" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="H1064" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="I1064" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J1064" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1064" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1.04 &lt;= EMA21 1.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D1065" t="n">
+        <v>558.26</v>
+      </c>
+      <c r="E1065" t="n">
+        <v>567.0700000000001</v>
+      </c>
+      <c r="F1065" t="n">
+        <v>567.0700000000001</v>
+      </c>
+      <c r="G1065" t="n">
+        <v>541.74</v>
+      </c>
+      <c r="H1065" t="n">
+        <v>533.9</v>
+      </c>
+      <c r="I1065" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J1065" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1065" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 558.26 &lt;= Upper 567.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="D1066" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="E1066" t="n">
+        <v>9.140000000000001</v>
+      </c>
+      <c r="F1066" t="n">
+        <v>9.140000000000001</v>
+      </c>
+      <c r="G1066" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="H1066" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="I1066" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J1066" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1066" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8.09 &lt;= EMA21 8.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D1067" t="n">
+        <v>108.09</v>
+      </c>
+      <c r="E1067" t="n">
+        <v>113.02</v>
+      </c>
+      <c r="F1067" t="n">
+        <v>113.02</v>
+      </c>
+      <c r="G1067" t="n">
+        <v>107.16</v>
+      </c>
+      <c r="H1067" t="n">
+        <v>107.62</v>
+      </c>
+      <c r="I1067" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J1067" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1067" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 107.16 &lt;= EMA21 107.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D1068" t="n">
+        <v>901.35</v>
+      </c>
+      <c r="E1068" t="n">
+        <v>977.5700000000001</v>
+      </c>
+      <c r="F1068" t="n">
+        <v>977.5700000000001</v>
+      </c>
+      <c r="G1068" t="n">
+        <v>914.21</v>
+      </c>
+      <c r="H1068" t="n">
+        <v>926.96</v>
+      </c>
+      <c r="I1068" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J1068" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1068" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 914.21 &lt;= EMA21 926.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="D1069" t="n">
+        <v>154.4</v>
+      </c>
+      <c r="E1069" t="n">
+        <v>170.09</v>
+      </c>
+      <c r="F1069" t="n">
+        <v>170.09</v>
+      </c>
+      <c r="G1069" t="n">
+        <v>158.48</v>
+      </c>
+      <c r="H1069" t="n">
+        <v>158.1</v>
+      </c>
+      <c r="I1069" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1069" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1069" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 154.40 &lt;= Upper 170.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D1070" t="n">
+        <v>305.48</v>
+      </c>
+      <c r="E1070" t="n">
+        <v>345.12</v>
+      </c>
+      <c r="F1070" t="n">
+        <v>345.12</v>
+      </c>
+      <c r="G1070" t="n">
+        <v>312.51</v>
+      </c>
+      <c r="H1070" t="n">
+        <v>320.5</v>
+      </c>
+      <c r="I1070" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1070" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1070" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 312.51 &lt;= EMA21 320.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D1071" t="n">
+        <v>194.61</v>
+      </c>
+      <c r="E1071" t="n">
+        <v>222.51</v>
+      </c>
+      <c r="F1071" t="n">
+        <v>222.51</v>
+      </c>
+      <c r="G1071" t="n">
+        <v>199.3</v>
+      </c>
+      <c r="H1071" t="n">
+        <v>204.29</v>
+      </c>
+      <c r="I1071" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J1071" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1071" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 199.30 &lt;= EMA21 204.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D1072" t="n">
+        <v>62.25</v>
+      </c>
+      <c r="E1072" t="n">
+        <v>61.05</v>
+      </c>
+      <c r="F1072" t="n">
+        <v>61.05</v>
+      </c>
+      <c r="G1072" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="H1072" t="n">
+        <v>58.27</v>
+      </c>
+      <c r="I1072" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="J1072" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1072" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="D1073" t="n">
+        <v>12.84</v>
+      </c>
+      <c r="E1073" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="F1073" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="G1073" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="H1073" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="I1073" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1073" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1073" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 12.84 &lt;= Upper 12.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="D1074" t="n">
+        <v>124.7</v>
+      </c>
+      <c r="E1074" t="n">
+        <v>133.15</v>
+      </c>
+      <c r="F1074" t="n">
+        <v>133.15</v>
+      </c>
+      <c r="G1074" t="n">
+        <v>126.45</v>
+      </c>
+      <c r="H1074" t="n">
+        <v>125.83</v>
+      </c>
+      <c r="I1074" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1074" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1074" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 124.70 &lt;= Upper 133.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D1075" t="n">
+        <v>112.79</v>
+      </c>
+      <c r="E1075" t="n">
+        <v>140.31</v>
+      </c>
+      <c r="F1075" t="n">
+        <v>140.31</v>
+      </c>
+      <c r="G1075" t="n">
+        <v>121</v>
+      </c>
+      <c r="H1075" t="n">
+        <v>124.79</v>
+      </c>
+      <c r="I1075" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J1075" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1075" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 121.00 &lt;= EMA21 124.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D1076" t="n">
+        <v>95.06</v>
+      </c>
+      <c r="E1076" t="n">
+        <v>97.48999999999999</v>
+      </c>
+      <c r="F1076" t="n">
+        <v>97.48999999999999</v>
+      </c>
+      <c r="G1076" t="n">
+        <v>92.59</v>
+      </c>
+      <c r="H1076" t="n">
+        <v>92.67</v>
+      </c>
+      <c r="I1076" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J1076" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1076" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 92.59 &lt;= EMA21 92.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D1077" t="n">
+        <v>226.26</v>
+      </c>
+      <c r="E1077" t="n">
+        <v>240.91</v>
+      </c>
+      <c r="F1077" t="n">
+        <v>240.91</v>
+      </c>
+      <c r="G1077" t="n">
+        <v>228.91</v>
+      </c>
+      <c r="H1077" t="n">
+        <v>231.97</v>
+      </c>
+      <c r="I1077" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J1077" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1077" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 228.91 &lt;= EMA21 231.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="D1078" t="n">
+        <v>124.6</v>
+      </c>
+      <c r="E1078" t="n">
+        <v>148.27</v>
+      </c>
+      <c r="F1078" t="n">
+        <v>148.27</v>
+      </c>
+      <c r="G1078" t="n">
+        <v>128.31</v>
+      </c>
+      <c r="H1078" t="n">
+        <v>134.53</v>
+      </c>
+      <c r="I1078" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1078" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1078" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 128.31 &lt;= EMA21 134.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D1079" t="n">
+        <v>36.22</v>
+      </c>
+      <c r="E1079" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="F1079" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="G1079" t="n">
+        <v>37.34</v>
+      </c>
+      <c r="H1079" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="I1079" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J1079" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1079" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 37.34 &lt;= EMA21 38.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D1080" t="n">
+        <v>98.37</v>
+      </c>
+      <c r="E1080" t="n">
+        <v>131.82</v>
+      </c>
+      <c r="F1080" t="n">
+        <v>131.82</v>
+      </c>
+      <c r="G1080" t="n">
+        <v>103.61</v>
+      </c>
+      <c r="H1080" t="n">
+        <v>109.86</v>
+      </c>
+      <c r="I1080" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J1080" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1080" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 103.61 &lt;= EMA21 109.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D1081" t="n">
+        <v>96.58</v>
+      </c>
+      <c r="E1081" t="n">
+        <v>111.38</v>
+      </c>
+      <c r="F1081" t="n">
+        <v>111.38</v>
+      </c>
+      <c r="G1081" t="n">
+        <v>100.66</v>
+      </c>
+      <c r="H1081" t="n">
+        <v>102.98</v>
+      </c>
+      <c r="I1081" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J1081" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1081" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 100.66 &lt;= EMA21 102.98)</t>
         </is>
       </c>
     </row>
@@ -42138,7 +46384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42855,6 +47101,161 @@
         <v>1.37</v>
       </c>
       <c r="G23" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" t="n">
+        <v>85.95</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>118.06</v>
+      </c>
+      <c r="E25" t="n">
+        <v>112.75</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>242.49</v>
+      </c>
+      <c r="E26" t="n">
+        <v>231.58</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>430.88</v>
+      </c>
+      <c r="E27" t="n">
+        <v>411.49</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>62.25</v>
+      </c>
+      <c r="E28" t="n">
+        <v>59.45</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -42952,19 +47353,19 @@
         <v>1961.07</v>
       </c>
       <c r="F2" t="n">
-        <v>665.6</v>
+        <v>670.24</v>
       </c>
       <c r="G2" t="n">
-        <v>1.82</v>
+        <v>2.53</v>
       </c>
       <c r="H2" t="n">
-        <v>638.51</v>
+        <v>648.3200000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>668.5999755859375</v>
+        <v>678.8699951171875</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -44895,7 +49296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45084,6 +49485,114 @@
       <c r="E7" t="inlineStr">
         <is>
           <t>Qualified breakout on IBM skipped: all slots full or insufficient cash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-16 05:01:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SKIPPED_CAPITAL_EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Qualified breakout on QRVO skipped: all slots full or insufficient cash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-16 05:01:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SKIPPED_CAPITAL_EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Qualified breakout on SWKS skipped: all slots full or insufficient cash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-16 05:01:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SKIPPED_CAPITAL_EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Qualified breakout on CRWD skipped: all slots full or insufficient cash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-16 05:01:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SKIPPED_CAPITAL_EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Qualified breakout on FFIV skipped: all slots full or insufficient cash.</t>
         </is>
       </c>
     </row>
@@ -45098,7 +49607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45610,6 +50119,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>05:01:30</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1689.8</v>
+      </c>
+      <c r="D16" t="n">
+        <v>7841.37</v>
+      </c>
+      <c r="E16" t="n">
+        <v>9531.17</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-468.83</v>
+      </c>
+      <c r="G16" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" t="n">
+        <v>10</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-17T05:09 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1081"/>
+  <dimension ref="A1:K1181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46370,6 +46370,4252 @@
       <c r="K1081" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 100.66 &lt;= EMA21 102.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D1082" t="n">
+        <v>332.41</v>
+      </c>
+      <c r="E1082" t="n">
+        <v>336.78</v>
+      </c>
+      <c r="F1082" t="n">
+        <v>336.78</v>
+      </c>
+      <c r="G1082" t="n">
+        <v>327.26</v>
+      </c>
+      <c r="H1082" t="n">
+        <v>322.16</v>
+      </c>
+      <c r="I1082" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J1082" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1082" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 332.41 &lt;= Upper 336.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D1083" t="n">
+        <v>490.3</v>
+      </c>
+      <c r="E1083" t="n">
+        <v>514.22</v>
+      </c>
+      <c r="F1083" t="n">
+        <v>514.22</v>
+      </c>
+      <c r="G1083" t="n">
+        <v>496.46</v>
+      </c>
+      <c r="H1083" t="n">
+        <v>491.93</v>
+      </c>
+      <c r="I1083" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J1083" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1083" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 490.30 &lt;= Upper 514.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D1084" t="n">
+        <v>213.9</v>
+      </c>
+      <c r="E1084" t="n">
+        <v>231.19</v>
+      </c>
+      <c r="F1084" t="n">
+        <v>231.19</v>
+      </c>
+      <c r="G1084" t="n">
+        <v>217.13</v>
+      </c>
+      <c r="H1084" t="n">
+        <v>217.76</v>
+      </c>
+      <c r="I1084" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1084" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1084" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 217.13 &lt;= EMA21 217.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D1085" t="n">
+        <v>342.87</v>
+      </c>
+      <c r="E1085" t="n">
+        <v>351.15</v>
+      </c>
+      <c r="F1085" t="n">
+        <v>351.15</v>
+      </c>
+      <c r="G1085" t="n">
+        <v>341.23</v>
+      </c>
+      <c r="H1085" t="n">
+        <v>341.94</v>
+      </c>
+      <c r="I1085" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J1085" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1085" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 341.23 &lt;= EMA21 341.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D1086" t="n">
+        <v>339.36</v>
+      </c>
+      <c r="E1086" t="n">
+        <v>347.37</v>
+      </c>
+      <c r="F1086" t="n">
+        <v>347.37</v>
+      </c>
+      <c r="G1086" t="n">
+        <v>338.02</v>
+      </c>
+      <c r="H1086" t="n">
+        <v>338.99</v>
+      </c>
+      <c r="I1086" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1086" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1086" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 338.02 &lt;= EMA21 338.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D1087" t="n">
+        <v>245.96</v>
+      </c>
+      <c r="E1087" t="n">
+        <v>267.54</v>
+      </c>
+      <c r="F1087" t="n">
+        <v>267.54</v>
+      </c>
+      <c r="G1087" t="n">
+        <v>252.64</v>
+      </c>
+      <c r="H1087" t="n">
+        <v>255.74</v>
+      </c>
+      <c r="I1087" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J1087" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1087" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 252.64 &lt;= EMA21 255.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D1088" t="n">
+        <v>673.3099999999999</v>
+      </c>
+      <c r="E1088" t="n">
+        <v>689.3200000000001</v>
+      </c>
+      <c r="F1088" t="n">
+        <v>689.3200000000001</v>
+      </c>
+      <c r="G1088" t="n">
+        <v>644.9</v>
+      </c>
+      <c r="H1088" t="n">
+        <v>618.74</v>
+      </c>
+      <c r="I1088" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J1088" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1088" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 673.31 &lt;= Upper 689.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D1089" t="n">
+        <v>358.08</v>
+      </c>
+      <c r="E1089" t="n">
+        <v>374.86</v>
+      </c>
+      <c r="F1089" t="n">
+        <v>374.86</v>
+      </c>
+      <c r="G1089" t="n">
+        <v>360.17</v>
+      </c>
+      <c r="H1089" t="n">
+        <v>356.64</v>
+      </c>
+      <c r="I1089" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J1089" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1089" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 358.08 &lt;= Upper 374.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D1090" t="n">
+        <v>339.51</v>
+      </c>
+      <c r="E1090" t="n">
+        <v>379.75</v>
+      </c>
+      <c r="F1090" t="n">
+        <v>379.75</v>
+      </c>
+      <c r="G1090" t="n">
+        <v>352.74</v>
+      </c>
+      <c r="H1090" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="I1090" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1090" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1090" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.74 &lt;= EMA21 363.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D1091" t="n">
+        <v>143.16</v>
+      </c>
+      <c r="E1091" t="n">
+        <v>162.02</v>
+      </c>
+      <c r="F1091" t="n">
+        <v>162.02</v>
+      </c>
+      <c r="G1091" t="n">
+        <v>148.14</v>
+      </c>
+      <c r="H1091" t="n">
+        <v>148.21</v>
+      </c>
+      <c r="I1091" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1091" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1091" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 148.14 &lt;= EMA21 148.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D1092" t="n">
+        <v>250.54</v>
+      </c>
+      <c r="E1092" t="n">
+        <v>285.18</v>
+      </c>
+      <c r="F1092" t="n">
+        <v>285.18</v>
+      </c>
+      <c r="G1092" t="n">
+        <v>250.4</v>
+      </c>
+      <c r="H1092" t="n">
+        <v>238.03</v>
+      </c>
+      <c r="I1092" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J1092" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1092" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 250.54 &lt;= Upper 285.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D1093" t="n">
+        <v>250.5</v>
+      </c>
+      <c r="E1093" t="n">
+        <v>299.21</v>
+      </c>
+      <c r="F1093" t="n">
+        <v>299.21</v>
+      </c>
+      <c r="G1093" t="n">
+        <v>260.28</v>
+      </c>
+      <c r="H1093" t="n">
+        <v>264.06</v>
+      </c>
+      <c r="I1093" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J1093" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1093" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 260.28 &lt;= EMA21 264.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D1094" t="n">
+        <v>512.5</v>
+      </c>
+      <c r="E1094" t="n">
+        <v>524.9400000000001</v>
+      </c>
+      <c r="F1094" t="n">
+        <v>524.9400000000001</v>
+      </c>
+      <c r="G1094" t="n">
+        <v>499.31</v>
+      </c>
+      <c r="H1094" t="n">
+        <v>491.23</v>
+      </c>
+      <c r="I1094" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J1094" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1094" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 512.50 &lt;= Upper 524.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D1095" t="n">
+        <v>101.05</v>
+      </c>
+      <c r="E1095" t="n">
+        <v>106.24</v>
+      </c>
+      <c r="F1095" t="n">
+        <v>106.24</v>
+      </c>
+      <c r="G1095" t="n">
+        <v>98.63</v>
+      </c>
+      <c r="H1095" t="n">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="I1095" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J1095" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1095" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 101.05 &lt;= Upper 106.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D1096" t="n">
+        <v>926.55</v>
+      </c>
+      <c r="E1096" t="n">
+        <v>1019.59</v>
+      </c>
+      <c r="F1096" t="n">
+        <v>1019.59</v>
+      </c>
+      <c r="G1096" t="n">
+        <v>953.0599999999999</v>
+      </c>
+      <c r="H1096" t="n">
+        <v>951.16</v>
+      </c>
+      <c r="I1096" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J1096" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1096" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 926.55 &lt;= Upper 1019.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D1097" t="n">
+        <v>184.84</v>
+      </c>
+      <c r="E1097" t="n">
+        <v>187.87</v>
+      </c>
+      <c r="F1097" t="n">
+        <v>187.87</v>
+      </c>
+      <c r="G1097" t="n">
+        <v>178.74</v>
+      </c>
+      <c r="H1097" t="n">
+        <v>172.79</v>
+      </c>
+      <c r="I1097" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J1097" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1097" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 184.84 &lt;= Upper 187.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="D1098" t="n">
+        <v>260.67</v>
+      </c>
+      <c r="E1098" t="n">
+        <v>269.62</v>
+      </c>
+      <c r="F1098" t="n">
+        <v>269.62</v>
+      </c>
+      <c r="G1098" t="n">
+        <v>261.75</v>
+      </c>
+      <c r="H1098" t="n">
+        <v>263.95</v>
+      </c>
+      <c r="I1098" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J1098" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1098" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 261.75 &lt;= EMA21 263.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D1099" t="n">
+        <v>415.38</v>
+      </c>
+      <c r="E1099" t="n">
+        <v>510.92</v>
+      </c>
+      <c r="F1099" t="n">
+        <v>510.92</v>
+      </c>
+      <c r="G1099" t="n">
+        <v>440.5</v>
+      </c>
+      <c r="H1099" t="n">
+        <v>462.02</v>
+      </c>
+      <c r="I1099" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1099" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1099" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 440.50 &lt;= EMA21 462.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D1100" t="n">
+        <v>269.23</v>
+      </c>
+      <c r="E1100" t="n">
+        <v>332.26</v>
+      </c>
+      <c r="F1100" t="n">
+        <v>332.26</v>
+      </c>
+      <c r="G1100" t="n">
+        <v>288.04</v>
+      </c>
+      <c r="H1100" t="n">
+        <v>298.66</v>
+      </c>
+      <c r="I1100" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1100" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1100" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 288.04 &lt;= EMA21 298.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D1101" t="n">
+        <v>167.36</v>
+      </c>
+      <c r="E1101" t="n">
+        <v>192.61</v>
+      </c>
+      <c r="F1101" t="n">
+        <v>192.61</v>
+      </c>
+      <c r="G1101" t="n">
+        <v>174.51</v>
+      </c>
+      <c r="H1101" t="n">
+        <v>180.52</v>
+      </c>
+      <c r="I1101" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J1101" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1101" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 174.51 &lt;= EMA21 180.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D1102" t="n">
+        <v>1602.22</v>
+      </c>
+      <c r="E1102" t="n">
+        <v>1814.15</v>
+      </c>
+      <c r="F1102" t="n">
+        <v>1814.15</v>
+      </c>
+      <c r="G1102" t="n">
+        <v>1651.79</v>
+      </c>
+      <c r="H1102" t="n">
+        <v>1689.34</v>
+      </c>
+      <c r="I1102" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J1102" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1102" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1651.79 &lt;= EMA21 1689.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D1103" t="n">
+        <v>362.04</v>
+      </c>
+      <c r="E1103" t="n">
+        <v>378.58</v>
+      </c>
+      <c r="F1103" t="n">
+        <v>378.58</v>
+      </c>
+      <c r="G1103" t="n">
+        <v>363.8</v>
+      </c>
+      <c r="H1103" t="n">
+        <v>366.49</v>
+      </c>
+      <c r="I1103" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1103" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1103" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.80 &lt;= EMA21 366.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D1104" t="n">
+        <v>229.71</v>
+      </c>
+      <c r="E1104" t="n">
+        <v>253.31</v>
+      </c>
+      <c r="F1104" t="n">
+        <v>253.31</v>
+      </c>
+      <c r="G1104" t="n">
+        <v>225.43</v>
+      </c>
+      <c r="H1104" t="n">
+        <v>224.05</v>
+      </c>
+      <c r="I1104" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1104" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1104" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 229.71 &lt;= Upper 253.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="D1105" t="n">
+        <v>218.98</v>
+      </c>
+      <c r="E1105" t="n">
+        <v>232.01</v>
+      </c>
+      <c r="F1105" t="n">
+        <v>232.01</v>
+      </c>
+      <c r="G1105" t="n">
+        <v>225.27</v>
+      </c>
+      <c r="H1105" t="n">
+        <v>228.09</v>
+      </c>
+      <c r="I1105" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1105" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1105" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 225.27 &lt;= EMA21 228.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D1106" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="E1106" t="n">
+        <v>77.33</v>
+      </c>
+      <c r="F1106" t="n">
+        <v>77.33</v>
+      </c>
+      <c r="G1106" t="n">
+        <v>71.64</v>
+      </c>
+      <c r="H1106" t="n">
+        <v>74</v>
+      </c>
+      <c r="I1106" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="J1106" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1106" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 71.64 &lt;= EMA21 74.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D1107" t="n">
+        <v>1147.61</v>
+      </c>
+      <c r="E1107" t="n">
+        <v>1357.17</v>
+      </c>
+      <c r="F1107" t="n">
+        <v>1357.17</v>
+      </c>
+      <c r="G1107" t="n">
+        <v>1187.73</v>
+      </c>
+      <c r="H1107" t="n">
+        <v>1236.24</v>
+      </c>
+      <c r="I1107" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J1107" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1107" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1187.73 &lt;= EMA21 1236.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D1108" t="n">
+        <v>85.59</v>
+      </c>
+      <c r="E1108" t="n">
+        <v>89.41</v>
+      </c>
+      <c r="F1108" t="n">
+        <v>89.41</v>
+      </c>
+      <c r="G1108" t="n">
+        <v>81.19</v>
+      </c>
+      <c r="H1108" t="n">
+        <v>75.59</v>
+      </c>
+      <c r="I1108" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J1108" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1108" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 85.59 &lt;= Upper 89.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D1109" t="n">
+        <v>113.97</v>
+      </c>
+      <c r="E1109" t="n">
+        <v>117.73</v>
+      </c>
+      <c r="F1109" t="n">
+        <v>117.73</v>
+      </c>
+      <c r="G1109" t="n">
+        <v>109.67</v>
+      </c>
+      <c r="H1109" t="n">
+        <v>104.06</v>
+      </c>
+      <c r="I1109" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="J1109" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1109" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 113.97 &lt;= Upper 117.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D1110" t="n">
+        <v>341.15</v>
+      </c>
+      <c r="E1110" t="n">
+        <v>395.49</v>
+      </c>
+      <c r="F1110" t="n">
+        <v>395.49</v>
+      </c>
+      <c r="G1110" t="n">
+        <v>351.79</v>
+      </c>
+      <c r="H1110" t="n">
+        <v>360.13</v>
+      </c>
+      <c r="I1110" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J1110" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1110" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 351.79 &lt;= EMA21 360.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>ENTG</t>
+        </is>
+      </c>
+      <c r="D1111" t="n">
+        <v>130.2</v>
+      </c>
+      <c r="E1111" t="n">
+        <v>148.94</v>
+      </c>
+      <c r="F1111" t="n">
+        <v>148.94</v>
+      </c>
+      <c r="G1111" t="n">
+        <v>134.28</v>
+      </c>
+      <c r="H1111" t="n">
+        <v>137.33</v>
+      </c>
+      <c r="I1111" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1111" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1111" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 134.28 &lt;= EMA21 137.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+      <c r="D1112" t="n">
+        <v>69.59</v>
+      </c>
+      <c r="E1112" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="F1112" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="G1112" t="n">
+        <v>72.06999999999999</v>
+      </c>
+      <c r="H1112" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="I1112" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J1112" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1112" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 72.07 &lt;= EMA21 73.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D1113" t="n">
+        <v>36.85</v>
+      </c>
+      <c r="E1113" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="F1113" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="G1113" t="n">
+        <v>37.51</v>
+      </c>
+      <c r="H1113" t="n">
+        <v>36.95</v>
+      </c>
+      <c r="I1113" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1113" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1113" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 36.85 &lt;= Upper 40.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D1114" t="n">
+        <v>563.29</v>
+      </c>
+      <c r="E1114" t="n">
+        <v>584.17</v>
+      </c>
+      <c r="F1114" t="n">
+        <v>584.17</v>
+      </c>
+      <c r="G1114" t="n">
+        <v>531.53</v>
+      </c>
+      <c r="H1114" t="n">
+        <v>502.36</v>
+      </c>
+      <c r="I1114" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J1114" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1114" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 563.29 &lt;= Upper 584.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D1115" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="E1115" t="n">
+        <v>35.05</v>
+      </c>
+      <c r="F1115" t="n">
+        <v>35.05</v>
+      </c>
+      <c r="G1115" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="H1115" t="n">
+        <v>31.47</v>
+      </c>
+      <c r="I1115" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1115" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1115" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 32.70 &lt;= Upper 35.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="D1116" t="n">
+        <v>416.97</v>
+      </c>
+      <c r="E1116" t="n">
+        <v>489.74</v>
+      </c>
+      <c r="F1116" t="n">
+        <v>489.74</v>
+      </c>
+      <c r="G1116" t="n">
+        <v>439.9</v>
+      </c>
+      <c r="H1116" t="n">
+        <v>455.28</v>
+      </c>
+      <c r="I1116" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J1116" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1116" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 439.90 &lt;= EMA21 455.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D1117" t="n">
+        <v>783.1799999999999</v>
+      </c>
+      <c r="E1117" t="n">
+        <v>896.66</v>
+      </c>
+      <c r="F1117" t="n">
+        <v>896.66</v>
+      </c>
+      <c r="G1117" t="n">
+        <v>818.36</v>
+      </c>
+      <c r="H1117" t="n">
+        <v>833.8200000000001</v>
+      </c>
+      <c r="I1117" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1117" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1117" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 818.36 &lt;= EMA21 833.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="D1118" t="n">
+        <v>197.54</v>
+      </c>
+      <c r="E1118" t="n">
+        <v>202.71</v>
+      </c>
+      <c r="F1118" t="n">
+        <v>202.71</v>
+      </c>
+      <c r="G1118" t="n">
+        <v>193.55</v>
+      </c>
+      <c r="H1118" t="n">
+        <v>192.39</v>
+      </c>
+      <c r="I1118" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1118" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1118" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 197.54 &lt;= Upper 202.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D1119" t="n">
+        <v>107.74</v>
+      </c>
+      <c r="E1119" t="n">
+        <v>112.68</v>
+      </c>
+      <c r="F1119" t="n">
+        <v>112.68</v>
+      </c>
+      <c r="G1119" t="n">
+        <v>109.52</v>
+      </c>
+      <c r="H1119" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="I1119" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J1119" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1119" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 109.52 &lt;= EMA21 110.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="D1120" t="n">
+        <v>189.64</v>
+      </c>
+      <c r="E1120" t="n">
+        <v>196.46</v>
+      </c>
+      <c r="F1120" t="n">
+        <v>196.46</v>
+      </c>
+      <c r="G1120" t="n">
+        <v>187.44</v>
+      </c>
+      <c r="H1120" t="n">
+        <v>183.72</v>
+      </c>
+      <c r="I1120" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1120" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1120" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 189.64 &lt;= Upper 196.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="D1121" t="n">
+        <v>237.49</v>
+      </c>
+      <c r="E1121" t="n">
+        <v>247</v>
+      </c>
+      <c r="F1121" t="n">
+        <v>247</v>
+      </c>
+      <c r="G1121" t="n">
+        <v>240.14</v>
+      </c>
+      <c r="H1121" t="n">
+        <v>237.42</v>
+      </c>
+      <c r="I1121" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J1121" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1121" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 237.49 &lt;= Upper 247.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D1122" t="n">
+        <v>139.82</v>
+      </c>
+      <c r="E1122" t="n">
+        <v>150.11</v>
+      </c>
+      <c r="F1122" t="n">
+        <v>150.11</v>
+      </c>
+      <c r="G1122" t="n">
+        <v>137.97</v>
+      </c>
+      <c r="H1122" t="n">
+        <v>134.21</v>
+      </c>
+      <c r="I1122" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J1122" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1122" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 139.82 &lt;= Upper 150.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D1123" t="n">
+        <v>318.13</v>
+      </c>
+      <c r="E1123" t="n">
+        <v>379.41</v>
+      </c>
+      <c r="F1123" t="n">
+        <v>379.41</v>
+      </c>
+      <c r="G1123" t="n">
+        <v>328.15</v>
+      </c>
+      <c r="H1123" t="n">
+        <v>333.02</v>
+      </c>
+      <c r="I1123" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J1123" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1123" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 328.15 &lt;= EMA21 333.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D1124" t="n">
+        <v>375.65</v>
+      </c>
+      <c r="E1124" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="F1124" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="G1124" t="n">
+        <v>357.4</v>
+      </c>
+      <c r="H1124" t="n">
+        <v>354.62</v>
+      </c>
+      <c r="I1124" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J1124" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1124" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 375.65 &lt;= Upper 390.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D1125" t="n">
+        <v>241.36</v>
+      </c>
+      <c r="E1125" t="n">
+        <v>246.23</v>
+      </c>
+      <c r="F1125" t="n">
+        <v>246.23</v>
+      </c>
+      <c r="G1125" t="n">
+        <v>224.46</v>
+      </c>
+      <c r="H1125" t="n">
+        <v>216.06</v>
+      </c>
+      <c r="I1125" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1125" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1125" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 241.36 &lt;= Upper 246.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D1126" t="n">
+        <v>331.02</v>
+      </c>
+      <c r="E1126" t="n">
+        <v>348.09</v>
+      </c>
+      <c r="F1126" t="n">
+        <v>348.09</v>
+      </c>
+      <c r="G1126" t="n">
+        <v>329.6</v>
+      </c>
+      <c r="H1126" t="n">
+        <v>326.08</v>
+      </c>
+      <c r="I1126" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1126" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1126" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 331.02 &lt;= Upper 348.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D1127" t="n">
+        <v>174.34</v>
+      </c>
+      <c r="E1127" t="n">
+        <v>187.99</v>
+      </c>
+      <c r="F1127" t="n">
+        <v>187.99</v>
+      </c>
+      <c r="G1127" t="n">
+        <v>172.72</v>
+      </c>
+      <c r="H1127" t="n">
+        <v>171.4</v>
+      </c>
+      <c r="I1127" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1127" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1127" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 174.34 &lt;= Upper 187.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D1128" t="n">
+        <v>230.79</v>
+      </c>
+      <c r="E1128" t="n">
+        <v>244.98</v>
+      </c>
+      <c r="F1128" t="n">
+        <v>244.98</v>
+      </c>
+      <c r="G1128" t="n">
+        <v>225.91</v>
+      </c>
+      <c r="H1128" t="n">
+        <v>229.36</v>
+      </c>
+      <c r="I1128" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J1128" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1128" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 225.91 &lt;= EMA21 229.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D1129" t="n">
+        <v>191.58</v>
+      </c>
+      <c r="E1129" t="n">
+        <v>197.71</v>
+      </c>
+      <c r="F1129" t="n">
+        <v>197.71</v>
+      </c>
+      <c r="G1129" t="n">
+        <v>180.59</v>
+      </c>
+      <c r="H1129" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="I1129" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1129" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1129" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 191.58 &lt;= Upper 197.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D1130" t="n">
+        <v>324.65</v>
+      </c>
+      <c r="E1130" t="n">
+        <v>332.87</v>
+      </c>
+      <c r="F1130" t="n">
+        <v>332.87</v>
+      </c>
+      <c r="G1130" t="n">
+        <v>312.13</v>
+      </c>
+      <c r="H1130" t="n">
+        <v>302.26</v>
+      </c>
+      <c r="I1130" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J1130" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1130" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 324.65 &lt;= Upper 332.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="D1131" t="n">
+        <v>376.34</v>
+      </c>
+      <c r="E1131" t="n">
+        <v>464.49</v>
+      </c>
+      <c r="F1131" t="n">
+        <v>464.49</v>
+      </c>
+      <c r="G1131" t="n">
+        <v>379.37</v>
+      </c>
+      <c r="H1131" t="n">
+        <v>388.85</v>
+      </c>
+      <c r="I1131" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1131" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1131" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 379.37 &lt;= EMA21 388.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D1132" t="n">
+        <v>171.77</v>
+      </c>
+      <c r="E1132" t="n">
+        <v>175.32</v>
+      </c>
+      <c r="F1132" t="n">
+        <v>175.32</v>
+      </c>
+      <c r="G1132" t="n">
+        <v>164.66</v>
+      </c>
+      <c r="H1132" t="n">
+        <v>161.78</v>
+      </c>
+      <c r="I1132" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1132" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1132" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 171.77 &lt;= Upper 175.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D1133" t="n">
+        <v>190.28</v>
+      </c>
+      <c r="E1133" t="n">
+        <v>200.16</v>
+      </c>
+      <c r="F1133" t="n">
+        <v>200.16</v>
+      </c>
+      <c r="G1133" t="n">
+        <v>185.86</v>
+      </c>
+      <c r="H1133" t="n">
+        <v>176.35</v>
+      </c>
+      <c r="I1133" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1133" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1133" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 190.28 &lt;= Upper 200.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>WDAY</t>
+        </is>
+      </c>
+      <c r="D1134" t="n">
+        <v>187.76</v>
+      </c>
+      <c r="E1134" t="n">
+        <v>207.49</v>
+      </c>
+      <c r="F1134" t="n">
+        <v>207.49</v>
+      </c>
+      <c r="G1134" t="n">
+        <v>190.69</v>
+      </c>
+      <c r="H1134" t="n">
+        <v>189.71</v>
+      </c>
+      <c r="I1134" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J1134" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1134" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 187.76 &lt;= Upper 207.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="D1135" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="E1135" t="n">
+        <v>264.34</v>
+      </c>
+      <c r="F1135" t="n">
+        <v>264.34</v>
+      </c>
+      <c r="G1135" t="n">
+        <v>239.33</v>
+      </c>
+      <c r="H1135" t="n">
+        <v>238.67</v>
+      </c>
+      <c r="I1135" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J1135" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1135" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 236.46 &lt;= Upper 264.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="D1136" t="n">
+        <v>264.9</v>
+      </c>
+      <c r="E1136" t="n">
+        <v>292.27</v>
+      </c>
+      <c r="F1136" t="n">
+        <v>292.27</v>
+      </c>
+      <c r="G1136" t="n">
+        <v>266.05</v>
+      </c>
+      <c r="H1136" t="n">
+        <v>259.85</v>
+      </c>
+      <c r="I1136" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J1136" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1136" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 264.90 &lt;= Upper 292.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D1137" t="n">
+        <v>91.94</v>
+      </c>
+      <c r="E1137" t="n">
+        <v>108.07</v>
+      </c>
+      <c r="F1137" t="n">
+        <v>108.07</v>
+      </c>
+      <c r="G1137" t="n">
+        <v>95.23</v>
+      </c>
+      <c r="H1137" t="n">
+        <v>97.23999999999999</v>
+      </c>
+      <c r="I1137" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J1137" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1137" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 95.23 &lt;= EMA21 97.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D1138" t="n">
+        <v>188.12</v>
+      </c>
+      <c r="E1138" t="n">
+        <v>201.08</v>
+      </c>
+      <c r="F1138" t="n">
+        <v>201.08</v>
+      </c>
+      <c r="G1138" t="n">
+        <v>177.15</v>
+      </c>
+      <c r="H1138" t="n">
+        <v>166.24</v>
+      </c>
+      <c r="I1138" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1138" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1138" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 188.12 &lt;= Upper 201.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="D1139" t="n">
+        <v>326.56</v>
+      </c>
+      <c r="E1139" t="n">
+        <v>332.79</v>
+      </c>
+      <c r="F1139" t="n">
+        <v>332.79</v>
+      </c>
+      <c r="G1139" t="n">
+        <v>322.56</v>
+      </c>
+      <c r="H1139" t="n">
+        <v>325.61</v>
+      </c>
+      <c r="I1139" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1139" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1139" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 322.56 &lt;= EMA21 325.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="D1140" t="n">
+        <v>468.42</v>
+      </c>
+      <c r="E1140" t="n">
+        <v>673.1</v>
+      </c>
+      <c r="F1140" t="n">
+        <v>673.1</v>
+      </c>
+      <c r="G1140" t="n">
+        <v>490.07</v>
+      </c>
+      <c r="H1140" t="n">
+        <v>524.5700000000001</v>
+      </c>
+      <c r="I1140" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="J1140" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1140" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 490.07 &lt;= EMA21 524.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="D1141" t="n">
+        <v>279.9</v>
+      </c>
+      <c r="E1141" t="n">
+        <v>353.74</v>
+      </c>
+      <c r="F1141" t="n">
+        <v>353.74</v>
+      </c>
+      <c r="G1141" t="n">
+        <v>288.13</v>
+      </c>
+      <c r="H1141" t="n">
+        <v>303.16</v>
+      </c>
+      <c r="I1141" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1141" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1141" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 288.13 &lt;= EMA21 303.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D1142" t="n">
+        <v>378.47</v>
+      </c>
+      <c r="E1142" t="n">
+        <v>451.19</v>
+      </c>
+      <c r="F1142" t="n">
+        <v>451.19</v>
+      </c>
+      <c r="G1142" t="n">
+        <v>390.01</v>
+      </c>
+      <c r="H1142" t="n">
+        <v>399.98</v>
+      </c>
+      <c r="I1142" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1142" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1142" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 390.01 &lt;= EMA21 399.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D1143" t="n">
+        <v>220.31</v>
+      </c>
+      <c r="E1143" t="n">
+        <v>277.84</v>
+      </c>
+      <c r="F1143" t="n">
+        <v>277.84</v>
+      </c>
+      <c r="G1143" t="n">
+        <v>224.33</v>
+      </c>
+      <c r="H1143" t="n">
+        <v>231.76</v>
+      </c>
+      <c r="I1143" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J1143" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1143" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 224.33 &lt;= EMA21 231.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="J1144" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1144" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D1145" t="n">
+        <v>131.16</v>
+      </c>
+      <c r="E1145" t="n">
+        <v>166.96</v>
+      </c>
+      <c r="F1145" t="n">
+        <v>166.96</v>
+      </c>
+      <c r="G1145" t="n">
+        <v>135.8</v>
+      </c>
+      <c r="H1145" t="n">
+        <v>140.37</v>
+      </c>
+      <c r="I1145" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J1145" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1145" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.80 &lt;= EMA21 140.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>TYL</t>
+        </is>
+      </c>
+      <c r="D1146" t="n">
+        <v>346.44</v>
+      </c>
+      <c r="E1146" t="n">
+        <v>384.81</v>
+      </c>
+      <c r="F1146" t="n">
+        <v>384.81</v>
+      </c>
+      <c r="G1146" t="n">
+        <v>351.38</v>
+      </c>
+      <c r="H1146" t="n">
+        <v>349.37</v>
+      </c>
+      <c r="I1146" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J1146" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1146" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 346.44 &lt;= Upper 384.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="D1147" t="n">
+        <v>147.32</v>
+      </c>
+      <c r="E1147" t="n">
+        <v>161.91</v>
+      </c>
+      <c r="F1147" t="n">
+        <v>161.91</v>
+      </c>
+      <c r="G1147" t="n">
+        <v>147.36</v>
+      </c>
+      <c r="H1147" t="n">
+        <v>147.86</v>
+      </c>
+      <c r="I1147" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J1147" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1147" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 147.36 &lt;= EMA21 147.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1148" t="n">
+        <v>191.57</v>
+      </c>
+      <c r="E1148" t="n">
+        <v>209.47</v>
+      </c>
+      <c r="F1148" t="n">
+        <v>209.47</v>
+      </c>
+      <c r="G1148" t="n">
+        <v>187.56</v>
+      </c>
+      <c r="H1148" t="n">
+        <v>185.48</v>
+      </c>
+      <c r="I1148" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J1148" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1148" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 191.57 &lt;= Upper 209.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D1149" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="E1149" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="F1149" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="G1149" t="n">
+        <v>61.78</v>
+      </c>
+      <c r="H1149" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="I1149" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1149" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1149" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 61.85 &lt;= Upper 65.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1150" t="n">
+        <v>11.08</v>
+      </c>
+      <c r="E1150" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F1150" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G1150" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="H1150" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="I1150" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1150" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1150" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11.34 &lt;= EMA21 11.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D1151" t="n">
+        <v>117.17</v>
+      </c>
+      <c r="E1151" t="n">
+        <v>124.28</v>
+      </c>
+      <c r="F1151" t="n">
+        <v>124.28</v>
+      </c>
+      <c r="G1151" t="n">
+        <v>118.17</v>
+      </c>
+      <c r="H1151" t="n">
+        <v>114.09</v>
+      </c>
+      <c r="I1151" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1151" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1151" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 117.17 &lt;= Upper 124.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>GEN</t>
+        </is>
+      </c>
+      <c r="D1152" t="n">
+        <v>30.65</v>
+      </c>
+      <c r="E1152" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="F1152" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="G1152" t="n">
+        <v>30.58</v>
+      </c>
+      <c r="H1152" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I1152" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J1152" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1152" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 30.65 &lt;= Upper 32.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D1153" t="n">
+        <v>149.96</v>
+      </c>
+      <c r="E1153" t="n">
+        <v>159.82</v>
+      </c>
+      <c r="F1153" t="n">
+        <v>159.82</v>
+      </c>
+      <c r="G1153" t="n">
+        <v>149.45</v>
+      </c>
+      <c r="H1153" t="n">
+        <v>146.45</v>
+      </c>
+      <c r="I1153" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J1153" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1153" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 149.96 &lt;= Upper 159.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D1154" t="n">
+        <v>423.59</v>
+      </c>
+      <c r="E1154" t="n">
+        <v>427.02</v>
+      </c>
+      <c r="F1154" t="n">
+        <v>427.02</v>
+      </c>
+      <c r="G1154" t="n">
+        <v>410.73</v>
+      </c>
+      <c r="H1154" t="n">
+        <v>404.19</v>
+      </c>
+      <c r="I1154" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="J1154" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1154" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 423.59 &lt;= Upper 427.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>JNPR</t>
+        </is>
+      </c>
+      <c r="J1155" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1155" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="D1156" t="n">
+        <v>104.48</v>
+      </c>
+      <c r="E1156" t="n">
+        <v>112.29</v>
+      </c>
+      <c r="F1156" t="n">
+        <v>112.29</v>
+      </c>
+      <c r="G1156" t="n">
+        <v>106.33</v>
+      </c>
+      <c r="H1156" t="n">
+        <v>108.68</v>
+      </c>
+      <c r="I1156" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J1156" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1156" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.33 &lt;= EMA21 108.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="J1157" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1157" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="D1158" t="n">
+        <v>211.81</v>
+      </c>
+      <c r="E1158" t="n">
+        <v>244.8</v>
+      </c>
+      <c r="F1158" t="n">
+        <v>244.8</v>
+      </c>
+      <c r="G1158" t="n">
+        <v>216.32</v>
+      </c>
+      <c r="H1158" t="n">
+        <v>222.67</v>
+      </c>
+      <c r="I1158" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1158" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1158" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 216.32 &lt;= EMA21 222.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D1159" t="n">
+        <v>47.43</v>
+      </c>
+      <c r="E1159" t="n">
+        <v>50.47</v>
+      </c>
+      <c r="F1159" t="n">
+        <v>50.47</v>
+      </c>
+      <c r="G1159" t="n">
+        <v>46.23</v>
+      </c>
+      <c r="H1159" t="n">
+        <v>43.78</v>
+      </c>
+      <c r="I1159" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1159" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1159" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 47.43 &lt;= Upper 50.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D1160" t="n">
+        <v>42.13</v>
+      </c>
+      <c r="E1160" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="F1160" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="G1160" t="n">
+        <v>42.76</v>
+      </c>
+      <c r="H1160" t="n">
+        <v>42.41</v>
+      </c>
+      <c r="I1160" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J1160" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1160" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 42.13 &lt;= Upper 47.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D1161" t="n">
+        <v>76.41</v>
+      </c>
+      <c r="E1161" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="F1161" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="G1161" t="n">
+        <v>78.09</v>
+      </c>
+      <c r="H1161" t="n">
+        <v>78.26000000000001</v>
+      </c>
+      <c r="I1161" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J1161" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1161" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 78.09 &lt;= EMA21 78.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D1162" t="n">
+        <v>106.99</v>
+      </c>
+      <c r="E1162" t="n">
+        <v>110.84</v>
+      </c>
+      <c r="F1162" t="n">
+        <v>110.84</v>
+      </c>
+      <c r="G1162" t="n">
+        <v>106.68</v>
+      </c>
+      <c r="H1162" t="n">
+        <v>106.11</v>
+      </c>
+      <c r="I1162" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J1162" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1162" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 106.99 &lt;= Upper 110.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="D1163" t="n">
+        <v>28.07</v>
+      </c>
+      <c r="E1163" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="F1163" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="G1163" t="n">
+        <v>28.14</v>
+      </c>
+      <c r="H1163" t="n">
+        <v>28.07</v>
+      </c>
+      <c r="I1163" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1163" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1163" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 28.07 &lt;= Upper 28.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="D1164" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E1164" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F1164" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G1164" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="H1164" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I1164" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J1164" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1164" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1.03 &lt;= EMA21 1.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D1165" t="n">
+        <v>547.4299999999999</v>
+      </c>
+      <c r="E1165" t="n">
+        <v>566.46</v>
+      </c>
+      <c r="F1165" t="n">
+        <v>566.46</v>
+      </c>
+      <c r="G1165" t="n">
+        <v>542.88</v>
+      </c>
+      <c r="H1165" t="n">
+        <v>535.13</v>
+      </c>
+      <c r="I1165" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J1165" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1165" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 547.43 &lt;= Upper 566.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="D1166" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="E1166" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="F1166" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="G1166" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="H1166" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="I1166" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J1166" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1166" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8.04 &lt;= EMA21 8.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D1167" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="E1167" t="n">
+        <v>111.35</v>
+      </c>
+      <c r="F1167" t="n">
+        <v>111.35</v>
+      </c>
+      <c r="G1167" t="n">
+        <v>107.23</v>
+      </c>
+      <c r="H1167" t="n">
+        <v>107.61</v>
+      </c>
+      <c r="I1167" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J1167" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1167" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 107.23 &lt;= EMA21 107.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D1168" t="n">
+        <v>893.74</v>
+      </c>
+      <c r="E1168" t="n">
+        <v>975.39</v>
+      </c>
+      <c r="F1168" t="n">
+        <v>975.39</v>
+      </c>
+      <c r="G1168" t="n">
+        <v>910.12</v>
+      </c>
+      <c r="H1168" t="n">
+        <v>923.9400000000001</v>
+      </c>
+      <c r="I1168" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J1168" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1168" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 910.12 &lt;= EMA21 923.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="D1169" t="n">
+        <v>154.68</v>
+      </c>
+      <c r="E1169" t="n">
+        <v>169.79</v>
+      </c>
+      <c r="F1169" t="n">
+        <v>169.79</v>
+      </c>
+      <c r="G1169" t="n">
+        <v>157.72</v>
+      </c>
+      <c r="H1169" t="n">
+        <v>157.79</v>
+      </c>
+      <c r="I1169" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J1169" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1169" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 157.72 &lt;= EMA21 157.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D1170" t="n">
+        <v>302.47</v>
+      </c>
+      <c r="E1170" t="n">
+        <v>344.39</v>
+      </c>
+      <c r="F1170" t="n">
+        <v>344.39</v>
+      </c>
+      <c r="G1170" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="H1170" t="n">
+        <v>318.86</v>
+      </c>
+      <c r="I1170" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1170" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1170" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 310.50 &lt;= EMA21 318.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D1171" t="n">
+        <v>194.1</v>
+      </c>
+      <c r="E1171" t="n">
+        <v>221.63</v>
+      </c>
+      <c r="F1171" t="n">
+        <v>221.63</v>
+      </c>
+      <c r="G1171" t="n">
+        <v>198.26</v>
+      </c>
+      <c r="H1171" t="n">
+        <v>203.36</v>
+      </c>
+      <c r="I1171" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1171" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1171" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 198.26 &lt;= EMA21 203.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D1172" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="E1172" t="n">
+        <v>61.48</v>
+      </c>
+      <c r="F1172" t="n">
+        <v>61.48</v>
+      </c>
+      <c r="G1172" t="n">
+        <v>59.51</v>
+      </c>
+      <c r="H1172" t="n">
+        <v>58.53</v>
+      </c>
+      <c r="I1172" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J1172" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1172" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 61.14 &lt;= Upper 61.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="D1173" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="E1173" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="F1173" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="G1173" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="H1173" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="I1173" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1173" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1173" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 12.56 &lt;= Upper 12.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="D1174" t="n">
+        <v>123.01</v>
+      </c>
+      <c r="E1174" t="n">
+        <v>133.02</v>
+      </c>
+      <c r="F1174" t="n">
+        <v>133.02</v>
+      </c>
+      <c r="G1174" t="n">
+        <v>125.76</v>
+      </c>
+      <c r="H1174" t="n">
+        <v>125.57</v>
+      </c>
+      <c r="I1174" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1174" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1174" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 123.01 &lt;= Upper 133.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D1175" t="n">
+        <v>112.4</v>
+      </c>
+      <c r="E1175" t="n">
+        <v>140.88</v>
+      </c>
+      <c r="F1175" t="n">
+        <v>140.88</v>
+      </c>
+      <c r="G1175" t="n">
+        <v>119.28</v>
+      </c>
+      <c r="H1175" t="n">
+        <v>123.67</v>
+      </c>
+      <c r="I1175" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J1175" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1175" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 119.28 &lt;= EMA21 123.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D1176" t="n">
+        <v>92.98</v>
+      </c>
+      <c r="E1176" t="n">
+        <v>97.51000000000001</v>
+      </c>
+      <c r="F1176" t="n">
+        <v>97.51000000000001</v>
+      </c>
+      <c r="G1176" t="n">
+        <v>92.67</v>
+      </c>
+      <c r="H1176" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="I1176" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J1176" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1176" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 92.67 &lt;= EMA21 92.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D1177" t="n">
+        <v>224.8</v>
+      </c>
+      <c r="E1177" t="n">
+        <v>240.54</v>
+      </c>
+      <c r="F1177" t="n">
+        <v>240.54</v>
+      </c>
+      <c r="G1177" t="n">
+        <v>228.09</v>
+      </c>
+      <c r="H1177" t="n">
+        <v>231.32</v>
+      </c>
+      <c r="I1177" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1177" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1177" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 228.09 &lt;= EMA21 231.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="D1178" t="n">
+        <v>122.84</v>
+      </c>
+      <c r="E1178" t="n">
+        <v>145.38</v>
+      </c>
+      <c r="F1178" t="n">
+        <v>145.38</v>
+      </c>
+      <c r="G1178" t="n">
+        <v>127.22</v>
+      </c>
+      <c r="H1178" t="n">
+        <v>133.47</v>
+      </c>
+      <c r="I1178" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1178" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1178" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 127.22 &lt;= EMA21 133.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D1179" t="n">
+        <v>35.78</v>
+      </c>
+      <c r="E1179" t="n">
+        <v>41.03</v>
+      </c>
+      <c r="F1179" t="n">
+        <v>41.03</v>
+      </c>
+      <c r="G1179" t="n">
+        <v>37.03</v>
+      </c>
+      <c r="H1179" t="n">
+        <v>38.15</v>
+      </c>
+      <c r="I1179" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1179" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1179" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 37.03 &lt;= EMA21 38.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D1180" t="n">
+        <v>95.98</v>
+      </c>
+      <c r="E1180" t="n">
+        <v>131.7</v>
+      </c>
+      <c r="F1180" t="n">
+        <v>131.7</v>
+      </c>
+      <c r="G1180" t="n">
+        <v>102.09</v>
+      </c>
+      <c r="H1180" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="I1180" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J1180" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1180" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 102.09 &lt;= EMA21 108.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D1181" t="n">
+        <v>97.34</v>
+      </c>
+      <c r="E1181" t="n">
+        <v>111.51</v>
+      </c>
+      <c r="F1181" t="n">
+        <v>111.51</v>
+      </c>
+      <c r="G1181" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1181" t="n">
+        <v>102.47</v>
+      </c>
+      <c r="I1181" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J1181" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1181" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 100.00 &lt;= EMA21 102.47)</t>
         </is>
       </c>
     </row>
@@ -47272,7 +51518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47353,19 +51599,19 @@
         <v>1961.07</v>
       </c>
       <c r="F2" t="n">
-        <v>670.24</v>
+        <v>673.3099999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>2.53</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>648.3200000000001</v>
+        <v>654.47</v>
       </c>
       <c r="I2" t="n">
-        <v>678.8699951171875</v>
+        <v>685.3099975585938</v>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -47376,7 +51622,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RBLX</t>
+          <t>NET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -47385,28 +51631,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>51.29</v>
+        <v>330.36</v>
       </c>
       <c r="D3" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>1949.02</v>
+        <v>1982.16</v>
       </c>
       <c r="F3" t="n">
-        <v>51.29</v>
+        <v>324.65</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>-1.73</v>
       </c>
       <c r="H3" t="n">
-        <v>48.98</v>
+        <v>319.51</v>
       </c>
       <c r="I3" t="n">
-        <v>51.29</v>
+        <v>334.5700073242188</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -47417,7 +51663,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -47426,71 +51672,30 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>330.36</v>
+        <v>60.91</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="E4" t="n">
-        <v>1982.16</v>
+        <v>1949.12</v>
       </c>
       <c r="F4" t="n">
-        <v>330.36</v>
+        <v>61.14</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.38</v>
       </c>
       <c r="H4" t="n">
-        <v>315.49</v>
+        <v>59.62</v>
       </c>
       <c r="I4" t="n">
-        <v>330.36</v>
+        <v>62.43000030517578</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>60.91</v>
-      </c>
-      <c r="D5" t="n">
-        <v>32</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1949.12</v>
-      </c>
-      <c r="F5" t="n">
-        <v>60.91</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>58.17</v>
-      </c>
-      <c r="I5" t="n">
-        <v>60.91</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -47507,7 +51712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48082,6 +52287,57 @@
         <v>1</v>
       </c>
       <c r="M11" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>51.29</v>
+      </c>
+      <c r="E12" t="n">
+        <v>48.98</v>
+      </c>
+      <c r="F12" t="n">
+        <v>38</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1949.02</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-4.504</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-4.554</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-88.76000000000001</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -48098,7 +52354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49282,6 +53538,55 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-17 05:09:07</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>761A03D483</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>48.98</v>
+      </c>
+      <c r="G25" t="n">
+        <v>48.98</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>38</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
         </is>
       </c>
     </row>
@@ -49607,7 +53912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50152,6 +54457,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>05:09:08</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3550.06</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5892.35</v>
+      </c>
+      <c r="E17" t="n">
+        <v>9442.41</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-557.59</v>
+      </c>
+      <c r="G17" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>11</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-18T05:03 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1181"/>
+  <dimension ref="A1:K1281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50616,6 +50616,4252 @@
       <c r="K1181" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 100.00 &lt;= EMA21 102.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D1182" t="n">
+        <v>337</v>
+      </c>
+      <c r="E1182" t="n">
+        <v>339.28</v>
+      </c>
+      <c r="F1182" t="n">
+        <v>339.28</v>
+      </c>
+      <c r="G1182" t="n">
+        <v>329.21</v>
+      </c>
+      <c r="H1182" t="n">
+        <v>323.51</v>
+      </c>
+      <c r="I1182" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1182" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1182" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 337.00 &lt;= Upper 339.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D1183" t="n">
+        <v>497.75</v>
+      </c>
+      <c r="E1183" t="n">
+        <v>513.92</v>
+      </c>
+      <c r="F1183" t="n">
+        <v>513.92</v>
+      </c>
+      <c r="G1183" t="n">
+        <v>496.72</v>
+      </c>
+      <c r="H1183" t="n">
+        <v>492.46</v>
+      </c>
+      <c r="I1183" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J1183" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1183" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 497.75 &lt;= Upper 513.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D1184" t="n">
+        <v>219.34</v>
+      </c>
+      <c r="E1184" t="n">
+        <v>231.28</v>
+      </c>
+      <c r="F1184" t="n">
+        <v>231.28</v>
+      </c>
+      <c r="G1184" t="n">
+        <v>217.57</v>
+      </c>
+      <c r="H1184" t="n">
+        <v>217.9</v>
+      </c>
+      <c r="I1184" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1184" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1184" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 217.57 &lt;= EMA21 217.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D1185" t="n">
+        <v>347.33</v>
+      </c>
+      <c r="E1185" t="n">
+        <v>351.57</v>
+      </c>
+      <c r="F1185" t="n">
+        <v>351.57</v>
+      </c>
+      <c r="G1185" t="n">
+        <v>342.45</v>
+      </c>
+      <c r="H1185" t="n">
+        <v>342.43</v>
+      </c>
+      <c r="I1185" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J1185" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1185" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 347.33 &lt;= Upper 351.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D1186" t="n">
+        <v>343.68</v>
+      </c>
+      <c r="E1186" t="n">
+        <v>347.7</v>
+      </c>
+      <c r="F1186" t="n">
+        <v>347.7</v>
+      </c>
+      <c r="G1186" t="n">
+        <v>339.15</v>
+      </c>
+      <c r="H1186" t="n">
+        <v>339.42</v>
+      </c>
+      <c r="I1186" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1186" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1186" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 339.15 &lt;= EMA21 339.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D1187" t="n">
+        <v>251.19</v>
+      </c>
+      <c r="E1187" t="n">
+        <v>266.29</v>
+      </c>
+      <c r="F1187" t="n">
+        <v>266.29</v>
+      </c>
+      <c r="G1187" t="n">
+        <v>252.35</v>
+      </c>
+      <c r="H1187" t="n">
+        <v>255.32</v>
+      </c>
+      <c r="I1187" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1187" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1187" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 252.35 &lt;= EMA21 255.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D1188" t="n">
+        <v>682.3099999999999</v>
+      </c>
+      <c r="E1188" t="n">
+        <v>699.02</v>
+      </c>
+      <c r="F1188" t="n">
+        <v>699.02</v>
+      </c>
+      <c r="G1188" t="n">
+        <v>652.39</v>
+      </c>
+      <c r="H1188" t="n">
+        <v>624.52</v>
+      </c>
+      <c r="I1188" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1188" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1188" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 682.31 &lt;= Upper 699.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D1189" t="n">
+        <v>366.2</v>
+      </c>
+      <c r="E1189" t="n">
+        <v>375.68</v>
+      </c>
+      <c r="F1189" t="n">
+        <v>375.68</v>
+      </c>
+      <c r="G1189" t="n">
+        <v>361.37</v>
+      </c>
+      <c r="H1189" t="n">
+        <v>357.51</v>
+      </c>
+      <c r="I1189" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1189" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1189" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 366.20 &lt;= Upper 375.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D1190" t="n">
+        <v>347.3</v>
+      </c>
+      <c r="E1190" t="n">
+        <v>379.82</v>
+      </c>
+      <c r="F1190" t="n">
+        <v>379.82</v>
+      </c>
+      <c r="G1190" t="n">
+        <v>351.65</v>
+      </c>
+      <c r="H1190" t="n">
+        <v>361.93</v>
+      </c>
+      <c r="I1190" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1190" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1190" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 351.65 &lt;= EMA21 361.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D1191" t="n">
+        <v>150.59</v>
+      </c>
+      <c r="E1191" t="n">
+        <v>162.16</v>
+      </c>
+      <c r="F1191" t="n">
+        <v>162.16</v>
+      </c>
+      <c r="G1191" t="n">
+        <v>148.63</v>
+      </c>
+      <c r="H1191" t="n">
+        <v>148.43</v>
+      </c>
+      <c r="I1191" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1191" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1191" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 150.59 &lt;= Upper 162.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D1192" t="n">
+        <v>242.85</v>
+      </c>
+      <c r="E1192" t="n">
+        <v>284.17</v>
+      </c>
+      <c r="F1192" t="n">
+        <v>284.17</v>
+      </c>
+      <c r="G1192" t="n">
+        <v>248.89</v>
+      </c>
+      <c r="H1192" t="n">
+        <v>238.47</v>
+      </c>
+      <c r="I1192" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1192" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1192" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 242.85 &lt;= Upper 284.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D1193" t="n">
+        <v>252.67</v>
+      </c>
+      <c r="E1193" t="n">
+        <v>299.39</v>
+      </c>
+      <c r="F1193" t="n">
+        <v>299.39</v>
+      </c>
+      <c r="G1193" t="n">
+        <v>258.76</v>
+      </c>
+      <c r="H1193" t="n">
+        <v>263.03</v>
+      </c>
+      <c r="I1193" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1193" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1193" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 258.76 &lt;= EMA21 263.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D1194" t="n">
+        <v>545.09</v>
+      </c>
+      <c r="E1194" t="n">
+        <v>536.53</v>
+      </c>
+      <c r="F1194" t="n">
+        <v>536.53</v>
+      </c>
+      <c r="G1194" t="n">
+        <v>508.46</v>
+      </c>
+      <c r="H1194" t="n">
+        <v>496.12</v>
+      </c>
+      <c r="I1194" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="J1194" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1194" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D1195" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="E1195" t="n">
+        <v>108.66</v>
+      </c>
+      <c r="F1195" t="n">
+        <v>108.66</v>
+      </c>
+      <c r="G1195" t="n">
+        <v>100.67</v>
+      </c>
+      <c r="H1195" t="n">
+        <v>98.16</v>
+      </c>
+      <c r="I1195" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="J1195" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1195" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D1196" t="n">
+        <v>977.5</v>
+      </c>
+      <c r="E1196" t="n">
+        <v>1021.72</v>
+      </c>
+      <c r="F1196" t="n">
+        <v>1021.72</v>
+      </c>
+      <c r="G1196" t="n">
+        <v>957.95</v>
+      </c>
+      <c r="H1196" t="n">
+        <v>953.55</v>
+      </c>
+      <c r="I1196" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1196" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1196" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 977.50 &lt;= Upper 1021.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D1197" t="n">
+        <v>188.71</v>
+      </c>
+      <c r="E1197" t="n">
+        <v>190.66</v>
+      </c>
+      <c r="F1197" t="n">
+        <v>190.66</v>
+      </c>
+      <c r="G1197" t="n">
+        <v>180.74</v>
+      </c>
+      <c r="H1197" t="n">
+        <v>174.24</v>
+      </c>
+      <c r="I1197" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J1197" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1197" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 188.71 &lt;= Upper 190.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="D1198" t="n">
+        <v>258.14</v>
+      </c>
+      <c r="E1198" t="n">
+        <v>268.68</v>
+      </c>
+      <c r="F1198" t="n">
+        <v>268.68</v>
+      </c>
+      <c r="G1198" t="n">
+        <v>261.03</v>
+      </c>
+      <c r="H1198" t="n">
+        <v>263.42</v>
+      </c>
+      <c r="I1198" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J1198" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1198" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 261.03 &lt;= EMA21 263.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D1199" t="n">
+        <v>417.4</v>
+      </c>
+      <c r="E1199" t="n">
+        <v>507.74</v>
+      </c>
+      <c r="F1199" t="n">
+        <v>507.74</v>
+      </c>
+      <c r="G1199" t="n">
+        <v>435.88</v>
+      </c>
+      <c r="H1199" t="n">
+        <v>457.97</v>
+      </c>
+      <c r="I1199" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J1199" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1199" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 435.88 &lt;= EMA21 457.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D1200" t="n">
+        <v>269.31</v>
+      </c>
+      <c r="E1200" t="n">
+        <v>333.19</v>
+      </c>
+      <c r="F1200" t="n">
+        <v>333.19</v>
+      </c>
+      <c r="G1200" t="n">
+        <v>284.29</v>
+      </c>
+      <c r="H1200" t="n">
+        <v>295.99</v>
+      </c>
+      <c r="I1200" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J1200" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1200" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 284.29 &lt;= EMA21 295.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D1201" t="n">
+        <v>168.98</v>
+      </c>
+      <c r="E1201" t="n">
+        <v>191.76</v>
+      </c>
+      <c r="F1201" t="n">
+        <v>191.76</v>
+      </c>
+      <c r="G1201" t="n">
+        <v>173.4</v>
+      </c>
+      <c r="H1201" t="n">
+        <v>179.47</v>
+      </c>
+      <c r="I1201" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1201" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1201" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 173.40 &lt;= EMA21 179.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D1202" t="n">
+        <v>1629.67</v>
+      </c>
+      <c r="E1202" t="n">
+        <v>1809.22</v>
+      </c>
+      <c r="F1202" t="n">
+        <v>1809.22</v>
+      </c>
+      <c r="G1202" t="n">
+        <v>1647.36</v>
+      </c>
+      <c r="H1202" t="n">
+        <v>1683.92</v>
+      </c>
+      <c r="I1202" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J1202" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1202" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1647.36 &lt;= EMA21 1683.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D1203" t="n">
+        <v>362.65</v>
+      </c>
+      <c r="E1203" t="n">
+        <v>377.74</v>
+      </c>
+      <c r="F1203" t="n">
+        <v>377.74</v>
+      </c>
+      <c r="G1203" t="n">
+        <v>363.57</v>
+      </c>
+      <c r="H1203" t="n">
+        <v>366.14</v>
+      </c>
+      <c r="I1203" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1203" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1203" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.57 &lt;= EMA21 366.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D1204" t="n">
+        <v>240.76</v>
+      </c>
+      <c r="E1204" t="n">
+        <v>253.8</v>
+      </c>
+      <c r="F1204" t="n">
+        <v>253.8</v>
+      </c>
+      <c r="G1204" t="n">
+        <v>228.49</v>
+      </c>
+      <c r="H1204" t="n">
+        <v>225.57</v>
+      </c>
+      <c r="I1204" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1204" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1204" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 240.76 &lt;= Upper 253.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="D1205" t="n">
+        <v>227.95</v>
+      </c>
+      <c r="E1205" t="n">
+        <v>231.2</v>
+      </c>
+      <c r="F1205" t="n">
+        <v>231.2</v>
+      </c>
+      <c r="G1205" t="n">
+        <v>225.15</v>
+      </c>
+      <c r="H1205" t="n">
+        <v>227.23</v>
+      </c>
+      <c r="I1205" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J1205" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1205" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 225.15 &lt;= EMA21 227.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D1206" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="E1206" t="n">
+        <v>77</v>
+      </c>
+      <c r="F1206" t="n">
+        <v>77</v>
+      </c>
+      <c r="G1206" t="n">
+        <v>70.97</v>
+      </c>
+      <c r="H1206" t="n">
+        <v>73.48</v>
+      </c>
+      <c r="I1206" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="J1206" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1206" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 70.97 &lt;= EMA21 73.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D1207" t="n">
+        <v>1169.58</v>
+      </c>
+      <c r="E1207" t="n">
+        <v>1351.25</v>
+      </c>
+      <c r="F1207" t="n">
+        <v>1351.25</v>
+      </c>
+      <c r="G1207" t="n">
+        <v>1184.1</v>
+      </c>
+      <c r="H1207" t="n">
+        <v>1230.18</v>
+      </c>
+      <c r="I1207" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J1207" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1207" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1184.10 &lt;= EMA21 1230.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D1208" t="n">
+        <v>91.31999999999999</v>
+      </c>
+      <c r="E1208" t="n">
+        <v>92.26000000000001</v>
+      </c>
+      <c r="F1208" t="n">
+        <v>92.26000000000001</v>
+      </c>
+      <c r="G1208" t="n">
+        <v>83.20999999999999</v>
+      </c>
+      <c r="H1208" t="n">
+        <v>77.02</v>
+      </c>
+      <c r="I1208" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1208" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1208" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 91.32 &lt;= Upper 92.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D1209" t="n">
+        <v>119.51</v>
+      </c>
+      <c r="E1209" t="n">
+        <v>120.49</v>
+      </c>
+      <c r="F1209" t="n">
+        <v>120.49</v>
+      </c>
+      <c r="G1209" t="n">
+        <v>111.64</v>
+      </c>
+      <c r="H1209" t="n">
+        <v>105.46</v>
+      </c>
+      <c r="I1209" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J1209" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1209" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 119.51 &lt;= Upper 120.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D1210" t="n">
+        <v>353.13</v>
+      </c>
+      <c r="E1210" t="n">
+        <v>393</v>
+      </c>
+      <c r="F1210" t="n">
+        <v>393</v>
+      </c>
+      <c r="G1210" t="n">
+        <v>352.06</v>
+      </c>
+      <c r="H1210" t="n">
+        <v>359.49</v>
+      </c>
+      <c r="I1210" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1210" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1210" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.06 &lt;= EMA21 359.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>ENTG</t>
+        </is>
+      </c>
+      <c r="D1211" t="n">
+        <v>134.67</v>
+      </c>
+      <c r="E1211" t="n">
+        <v>148.05</v>
+      </c>
+      <c r="F1211" t="n">
+        <v>148.05</v>
+      </c>
+      <c r="G1211" t="n">
+        <v>134.36</v>
+      </c>
+      <c r="H1211" t="n">
+        <v>137.09</v>
+      </c>
+      <c r="I1211" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1211" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1211" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 134.36 &lt;= EMA21 137.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+      <c r="D1212" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="E1212" t="n">
+        <v>76.33</v>
+      </c>
+      <c r="F1212" t="n">
+        <v>76.33</v>
+      </c>
+      <c r="G1212" t="n">
+        <v>71.81999999999999</v>
+      </c>
+      <c r="H1212" t="n">
+        <v>73.44</v>
+      </c>
+      <c r="I1212" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J1212" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1212" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 71.82 &lt;= EMA21 73.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D1213" t="n">
+        <v>40.35</v>
+      </c>
+      <c r="E1213" t="n">
+        <v>40.71</v>
+      </c>
+      <c r="F1213" t="n">
+        <v>40.71</v>
+      </c>
+      <c r="G1213" t="n">
+        <v>38.07</v>
+      </c>
+      <c r="H1213" t="n">
+        <v>37.26</v>
+      </c>
+      <c r="I1213" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J1213" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1213" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 40.35 &lt;= Upper 40.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D1214" t="n">
+        <v>588.4</v>
+      </c>
+      <c r="E1214" t="n">
+        <v>598.12</v>
+      </c>
+      <c r="F1214" t="n">
+        <v>598.12</v>
+      </c>
+      <c r="G1214" t="n">
+        <v>542.9</v>
+      </c>
+      <c r="H1214" t="n">
+        <v>510.18</v>
+      </c>
+      <c r="I1214" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1214" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1214" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 588.40 &lt;= Upper 598.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D1215" t="n">
+        <v>34.66</v>
+      </c>
+      <c r="E1215" t="n">
+        <v>35.52</v>
+      </c>
+      <c r="F1215" t="n">
+        <v>35.52</v>
+      </c>
+      <c r="G1215" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="H1215" t="n">
+        <v>31.76</v>
+      </c>
+      <c r="I1215" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1215" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1215" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 34.66 &lt;= Upper 35.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="D1216" t="n">
+        <v>423.87</v>
+      </c>
+      <c r="E1216" t="n">
+        <v>489.62</v>
+      </c>
+      <c r="F1216" t="n">
+        <v>489.62</v>
+      </c>
+      <c r="G1216" t="n">
+        <v>436.7</v>
+      </c>
+      <c r="H1216" t="n">
+        <v>452.43</v>
+      </c>
+      <c r="I1216" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J1216" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1216" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 436.70 &lt;= EMA21 452.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D1217" t="n">
+        <v>803.13</v>
+      </c>
+      <c r="E1217" t="n">
+        <v>896.33</v>
+      </c>
+      <c r="F1217" t="n">
+        <v>896.33</v>
+      </c>
+      <c r="G1217" t="n">
+        <v>815.3099999999999</v>
+      </c>
+      <c r="H1217" t="n">
+        <v>831.03</v>
+      </c>
+      <c r="I1217" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J1217" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1217" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 815.31 &lt;= EMA21 831.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="D1218" t="n">
+        <v>199.53</v>
+      </c>
+      <c r="E1218" t="n">
+        <v>203.44</v>
+      </c>
+      <c r="F1218" t="n">
+        <v>203.44</v>
+      </c>
+      <c r="G1218" t="n">
+        <v>194.75</v>
+      </c>
+      <c r="H1218" t="n">
+        <v>193.04</v>
+      </c>
+      <c r="I1218" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J1218" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1218" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 199.53 &lt;= Upper 203.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D1219" t="n">
+        <v>110.24</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>112.65</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>112.65</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>109.67</v>
+      </c>
+      <c r="H1219" t="n">
+        <v>110.66</v>
+      </c>
+      <c r="I1219" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1219" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1219" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 109.67 &lt;= EMA21 110.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="D1220" t="n">
+        <v>190.29</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>196.88</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>196.88</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>188.01</v>
+      </c>
+      <c r="H1220" t="n">
+        <v>184.32</v>
+      </c>
+      <c r="I1220" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J1220" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1220" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 190.29 &lt;= Upper 196.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="D1221" t="n">
+        <v>237.75</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>247.04</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>247.04</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>239.66</v>
+      </c>
+      <c r="H1221" t="n">
+        <v>237.45</v>
+      </c>
+      <c r="I1221" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J1221" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1221" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 237.75 &lt;= Upper 247.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D1222" t="n">
+        <v>138.47</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>150.12</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>150.12</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>138.07</v>
+      </c>
+      <c r="H1222" t="n">
+        <v>134.59</v>
+      </c>
+      <c r="I1222" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J1222" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1222" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 138.47 &lt;= Upper 150.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D1223" t="n">
+        <v>313.13</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>377.88</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>377.88</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>325.15</v>
+      </c>
+      <c r="H1223" t="n">
+        <v>331.22</v>
+      </c>
+      <c r="I1223" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J1223" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1223" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 325.15 &lt;= EMA21 331.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D1224" t="n">
+        <v>375.06</v>
+      </c>
+      <c r="E1224" t="n">
+        <v>392.5</v>
+      </c>
+      <c r="F1224" t="n">
+        <v>392.5</v>
+      </c>
+      <c r="G1224" t="n">
+        <v>360.93</v>
+      </c>
+      <c r="H1224" t="n">
+        <v>356.48</v>
+      </c>
+      <c r="I1224" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J1224" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1224" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 375.06 &lt;= Upper 392.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D1225" t="n">
+        <v>245.7</v>
+      </c>
+      <c r="E1225" t="n">
+        <v>251.31</v>
+      </c>
+      <c r="F1225" t="n">
+        <v>251.31</v>
+      </c>
+      <c r="G1225" t="n">
+        <v>228.71</v>
+      </c>
+      <c r="H1225" t="n">
+        <v>218.76</v>
+      </c>
+      <c r="I1225" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J1225" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1225" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 245.70 &lt;= Upper 251.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D1226" t="n">
+        <v>338.39</v>
+      </c>
+      <c r="E1226" t="n">
+        <v>349.26</v>
+      </c>
+      <c r="F1226" t="n">
+        <v>349.26</v>
+      </c>
+      <c r="G1226" t="n">
+        <v>331.36</v>
+      </c>
+      <c r="H1226" t="n">
+        <v>327.2</v>
+      </c>
+      <c r="I1226" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1226" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1226" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 338.39 &lt;= Upper 349.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D1227" t="n">
+        <v>176.24</v>
+      </c>
+      <c r="E1227" t="n">
+        <v>188.05</v>
+      </c>
+      <c r="F1227" t="n">
+        <v>188.05</v>
+      </c>
+      <c r="G1227" t="n">
+        <v>173.42</v>
+      </c>
+      <c r="H1227" t="n">
+        <v>171.84</v>
+      </c>
+      <c r="I1227" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1227" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1227" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 176.24 &lt;= Upper 188.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D1228" t="n">
+        <v>236</v>
+      </c>
+      <c r="E1228" t="n">
+        <v>245.34</v>
+      </c>
+      <c r="F1228" t="n">
+        <v>245.34</v>
+      </c>
+      <c r="G1228" t="n">
+        <v>227.93</v>
+      </c>
+      <c r="H1228" t="n">
+        <v>229.96</v>
+      </c>
+      <c r="I1228" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1228" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1228" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 227.93 &lt;= EMA21 229.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D1229" t="n">
+        <v>197.47</v>
+      </c>
+      <c r="E1229" t="n">
+        <v>200.06</v>
+      </c>
+      <c r="F1229" t="n">
+        <v>200.06</v>
+      </c>
+      <c r="G1229" t="n">
+        <v>183.97</v>
+      </c>
+      <c r="H1229" t="n">
+        <v>178.41</v>
+      </c>
+      <c r="I1229" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J1229" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1229" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 197.47 &lt;= Upper 200.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D1230" t="n">
+        <v>333.94</v>
+      </c>
+      <c r="E1230" t="n">
+        <v>338.47</v>
+      </c>
+      <c r="F1230" t="n">
+        <v>338.47</v>
+      </c>
+      <c r="G1230" t="n">
+        <v>316.49</v>
+      </c>
+      <c r="H1230" t="n">
+        <v>305.14</v>
+      </c>
+      <c r="I1230" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1230" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1230" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 333.94 &lt;= Upper 338.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="D1231" t="n">
+        <v>393.42</v>
+      </c>
+      <c r="E1231" t="n">
+        <v>459.25</v>
+      </c>
+      <c r="F1231" t="n">
+        <v>459.25</v>
+      </c>
+      <c r="G1231" t="n">
+        <v>382.18</v>
+      </c>
+      <c r="H1231" t="n">
+        <v>389.26</v>
+      </c>
+      <c r="I1231" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1231" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1231" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 382.18 &lt;= EMA21 389.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D1232" t="n">
+        <v>172.58</v>
+      </c>
+      <c r="E1232" t="n">
+        <v>176.86</v>
+      </c>
+      <c r="F1232" t="n">
+        <v>176.86</v>
+      </c>
+      <c r="G1232" t="n">
+        <v>166.24</v>
+      </c>
+      <c r="H1232" t="n">
+        <v>162.76</v>
+      </c>
+      <c r="I1232" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J1232" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1232" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 172.58 &lt;= Upper 176.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D1233" t="n">
+        <v>192.53</v>
+      </c>
+      <c r="E1233" t="n">
+        <v>201.25</v>
+      </c>
+      <c r="F1233" t="n">
+        <v>201.25</v>
+      </c>
+      <c r="G1233" t="n">
+        <v>187.2</v>
+      </c>
+      <c r="H1233" t="n">
+        <v>177.82</v>
+      </c>
+      <c r="I1233" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J1233" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1233" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 192.53 &lt;= Upper 201.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>WDAY</t>
+        </is>
+      </c>
+      <c r="D1234" t="n">
+        <v>199.28</v>
+      </c>
+      <c r="E1234" t="n">
+        <v>207.59</v>
+      </c>
+      <c r="F1234" t="n">
+        <v>207.59</v>
+      </c>
+      <c r="G1234" t="n">
+        <v>192.41</v>
+      </c>
+      <c r="H1234" t="n">
+        <v>190.58</v>
+      </c>
+      <c r="I1234" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J1234" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1234" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 199.28 &lt;= Upper 207.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="D1235" t="n">
+        <v>229.58</v>
+      </c>
+      <c r="E1235" t="n">
+        <v>264.61</v>
+      </c>
+      <c r="F1235" t="n">
+        <v>264.61</v>
+      </c>
+      <c r="G1235" t="n">
+        <v>237.38</v>
+      </c>
+      <c r="H1235" t="n">
+        <v>237.84</v>
+      </c>
+      <c r="I1235" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J1235" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1235" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 237.38 &lt;= EMA21 237.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="D1236" t="n">
+        <v>263.75</v>
+      </c>
+      <c r="E1236" t="n">
+        <v>292.12</v>
+      </c>
+      <c r="F1236" t="n">
+        <v>292.12</v>
+      </c>
+      <c r="G1236" t="n">
+        <v>265.59</v>
+      </c>
+      <c r="H1236" t="n">
+        <v>260.21</v>
+      </c>
+      <c r="I1236" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J1236" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1236" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 263.75 &lt;= Upper 292.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D1237" t="n">
+        <v>92.16</v>
+      </c>
+      <c r="E1237" t="n">
+        <v>106.72</v>
+      </c>
+      <c r="F1237" t="n">
+        <v>106.72</v>
+      </c>
+      <c r="G1237" t="n">
+        <v>94.61</v>
+      </c>
+      <c r="H1237" t="n">
+        <v>96.77</v>
+      </c>
+      <c r="I1237" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J1237" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1237" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 94.61 &lt;= EMA21 96.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D1238" t="n">
+        <v>190.02</v>
+      </c>
+      <c r="E1238" t="n">
+        <v>204.24</v>
+      </c>
+      <c r="F1238" t="n">
+        <v>204.24</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>179.72</v>
+      </c>
+      <c r="H1238" t="n">
+        <v>168.4</v>
+      </c>
+      <c r="I1238" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1238" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1238" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 190.02 &lt;= Upper 204.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="D1239" t="n">
+        <v>321.6</v>
+      </c>
+      <c r="E1239" t="n">
+        <v>333.46</v>
+      </c>
+      <c r="F1239" t="n">
+        <v>333.46</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>322.37</v>
+      </c>
+      <c r="H1239" t="n">
+        <v>325.24</v>
+      </c>
+      <c r="I1239" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1239" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1239" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 322.37 &lt;= EMA21 325.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="D1240" t="n">
+        <v>453.5</v>
+      </c>
+      <c r="E1240" t="n">
+        <v>660.75</v>
+      </c>
+      <c r="F1240" t="n">
+        <v>660.75</v>
+      </c>
+      <c r="G1240" t="n">
+        <v>482.76</v>
+      </c>
+      <c r="H1240" t="n">
+        <v>518.11</v>
+      </c>
+      <c r="I1240" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1240" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1240" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 482.76 &lt;= EMA21 518.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="D1241" t="n">
+        <v>280.76</v>
+      </c>
+      <c r="E1241" t="n">
+        <v>353.38</v>
+      </c>
+      <c r="F1241" t="n">
+        <v>353.38</v>
+      </c>
+      <c r="G1241" t="n">
+        <v>286.66</v>
+      </c>
+      <c r="H1241" t="n">
+        <v>301.12</v>
+      </c>
+      <c r="I1241" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J1241" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1241" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 286.66 &lt;= EMA21 301.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D1242" t="n">
+        <v>381.17</v>
+      </c>
+      <c r="E1242" t="n">
+        <v>451.42</v>
+      </c>
+      <c r="F1242" t="n">
+        <v>451.42</v>
+      </c>
+      <c r="G1242" t="n">
+        <v>388.24</v>
+      </c>
+      <c r="H1242" t="n">
+        <v>398.27</v>
+      </c>
+      <c r="I1242" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1242" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1242" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 388.24 &lt;= EMA21 398.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D1243" t="n">
+        <v>218.64</v>
+      </c>
+      <c r="E1243" t="n">
+        <v>276.67</v>
+      </c>
+      <c r="F1243" t="n">
+        <v>276.67</v>
+      </c>
+      <c r="G1243" t="n">
+        <v>223.19</v>
+      </c>
+      <c r="H1243" t="n">
+        <v>230.57</v>
+      </c>
+      <c r="I1243" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J1243" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1243" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 223.19 &lt;= EMA21 230.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="J1244" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1244" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D1245" t="n">
+        <v>134.44</v>
+      </c>
+      <c r="E1245" t="n">
+        <v>166.3</v>
+      </c>
+      <c r="F1245" t="n">
+        <v>166.3</v>
+      </c>
+      <c r="G1245" t="n">
+        <v>135.53</v>
+      </c>
+      <c r="H1245" t="n">
+        <v>139.83</v>
+      </c>
+      <c r="I1245" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1245" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1245" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.53 &lt;= EMA21 139.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>TYL</t>
+        </is>
+      </c>
+      <c r="D1246" t="n">
+        <v>341.57</v>
+      </c>
+      <c r="E1246" t="n">
+        <v>385.05</v>
+      </c>
+      <c r="F1246" t="n">
+        <v>385.05</v>
+      </c>
+      <c r="G1246" t="n">
+        <v>349.42</v>
+      </c>
+      <c r="H1246" t="n">
+        <v>348.66</v>
+      </c>
+      <c r="I1246" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J1246" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1246" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 341.57 &lt;= Upper 385.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="D1247" t="n">
+        <v>146.23</v>
+      </c>
+      <c r="E1247" t="n">
+        <v>161.94</v>
+      </c>
+      <c r="F1247" t="n">
+        <v>161.94</v>
+      </c>
+      <c r="G1247" t="n">
+        <v>147.13</v>
+      </c>
+      <c r="H1247" t="n">
+        <v>147.71</v>
+      </c>
+      <c r="I1247" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J1247" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1247" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 147.13 &lt;= EMA21 147.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1248" t="n">
+        <v>187.8</v>
+      </c>
+      <c r="E1248" t="n">
+        <v>209.2</v>
+      </c>
+      <c r="F1248" t="n">
+        <v>209.2</v>
+      </c>
+      <c r="G1248" t="n">
+        <v>187.61</v>
+      </c>
+      <c r="H1248" t="n">
+        <v>185.69</v>
+      </c>
+      <c r="I1248" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1248" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1248" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 187.80 &lt;= Upper 209.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D1249" t="n">
+        <v>61.88</v>
+      </c>
+      <c r="E1249" t="n">
+        <v>66</v>
+      </c>
+      <c r="F1249" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1249" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="H1249" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="I1249" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J1249" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1249" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 61.88 &lt;= Upper 66.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1250" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="E1250" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="F1250" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="G1250" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="H1250" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="I1250" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J1250" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1250" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11.29 &lt;= EMA21 11.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D1251" t="n">
+        <v>117.1</v>
+      </c>
+      <c r="E1251" t="n">
+        <v>124.09</v>
+      </c>
+      <c r="F1251" t="n">
+        <v>124.09</v>
+      </c>
+      <c r="G1251" t="n">
+        <v>117.96</v>
+      </c>
+      <c r="H1251" t="n">
+        <v>114.37</v>
+      </c>
+      <c r="I1251" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J1251" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1251" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 117.10 &lt;= Upper 124.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>GEN</t>
+        </is>
+      </c>
+      <c r="D1252" t="n">
+        <v>30.21</v>
+      </c>
+      <c r="E1252" t="n">
+        <v>31.91</v>
+      </c>
+      <c r="F1252" t="n">
+        <v>31.91</v>
+      </c>
+      <c r="G1252" t="n">
+        <v>30.51</v>
+      </c>
+      <c r="H1252" t="n">
+        <v>30</v>
+      </c>
+      <c r="I1252" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1252" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1252" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 30.21 &lt;= Upper 31.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D1253" t="n">
+        <v>149.2</v>
+      </c>
+      <c r="E1253" t="n">
+        <v>159.86</v>
+      </c>
+      <c r="F1253" t="n">
+        <v>159.86</v>
+      </c>
+      <c r="G1253" t="n">
+        <v>149.4</v>
+      </c>
+      <c r="H1253" t="n">
+        <v>146.7</v>
+      </c>
+      <c r="I1253" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J1253" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1253" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 149.20 &lt;= Upper 159.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D1254" t="n">
+        <v>434.62</v>
+      </c>
+      <c r="E1254" t="n">
+        <v>432.97</v>
+      </c>
+      <c r="F1254" t="n">
+        <v>432.97</v>
+      </c>
+      <c r="G1254" t="n">
+        <v>415.51</v>
+      </c>
+      <c r="H1254" t="n">
+        <v>406.96</v>
+      </c>
+      <c r="I1254" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1254" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1254" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.07x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>JNPR</t>
+        </is>
+      </c>
+      <c r="J1255" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1255" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="D1256" t="n">
+        <v>107.08</v>
+      </c>
+      <c r="E1256" t="n">
+        <v>111.28</v>
+      </c>
+      <c r="F1256" t="n">
+        <v>111.28</v>
+      </c>
+      <c r="G1256" t="n">
+        <v>106.48</v>
+      </c>
+      <c r="H1256" t="n">
+        <v>108.53</v>
+      </c>
+      <c r="I1256" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J1256" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1256" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.48 &lt;= EMA21 108.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="J1257" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1257" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="D1258" t="n">
+        <v>210.62</v>
+      </c>
+      <c r="E1258" t="n">
+        <v>243.22</v>
+      </c>
+      <c r="F1258" t="n">
+        <v>243.22</v>
+      </c>
+      <c r="G1258" t="n">
+        <v>215.18</v>
+      </c>
+      <c r="H1258" t="n">
+        <v>221.57</v>
+      </c>
+      <c r="I1258" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1258" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1258" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 215.18 &lt;= EMA21 221.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D1259" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="E1259" t="n">
+        <v>51.06</v>
+      </c>
+      <c r="F1259" t="n">
+        <v>51.06</v>
+      </c>
+      <c r="G1259" t="n">
+        <v>46.48</v>
+      </c>
+      <c r="H1259" t="n">
+        <v>44.12</v>
+      </c>
+      <c r="I1259" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J1259" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1259" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 47.50 &lt;= Upper 51.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D1260" t="n">
+        <v>41.84</v>
+      </c>
+      <c r="E1260" t="n">
+        <v>46.81</v>
+      </c>
+      <c r="F1260" t="n">
+        <v>46.81</v>
+      </c>
+      <c r="G1260" t="n">
+        <v>42.58</v>
+      </c>
+      <c r="H1260" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="I1260" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J1260" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1260" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 41.84 &lt;= Upper 46.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D1261" t="n">
+        <v>75.31</v>
+      </c>
+      <c r="E1261" t="n">
+        <v>84.12</v>
+      </c>
+      <c r="F1261" t="n">
+        <v>84.12</v>
+      </c>
+      <c r="G1261" t="n">
+        <v>77.54000000000001</v>
+      </c>
+      <c r="H1261" t="n">
+        <v>77.98999999999999</v>
+      </c>
+      <c r="I1261" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J1261" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1261" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 77.54 &lt;= EMA21 77.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D1262" t="n">
+        <v>105.35</v>
+      </c>
+      <c r="E1262" t="n">
+        <v>110.86</v>
+      </c>
+      <c r="F1262" t="n">
+        <v>110.86</v>
+      </c>
+      <c r="G1262" t="n">
+        <v>106.42</v>
+      </c>
+      <c r="H1262" t="n">
+        <v>106.05</v>
+      </c>
+      <c r="I1262" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1262" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1262" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 105.35 &lt;= Upper 110.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="D1263" t="n">
+        <v>28.24</v>
+      </c>
+      <c r="E1263" t="n">
+        <v>28.98</v>
+      </c>
+      <c r="F1263" t="n">
+        <v>28.98</v>
+      </c>
+      <c r="G1263" t="n">
+        <v>28.16</v>
+      </c>
+      <c r="H1263" t="n">
+        <v>28.08</v>
+      </c>
+      <c r="I1263" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1263" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1263" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 28.24 &lt;= Upper 28.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="D1264" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E1264" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F1264" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G1264" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="H1264" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="I1264" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1264" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1264" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1.01 &lt;= EMA21 1.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D1265" t="n">
+        <v>528.84</v>
+      </c>
+      <c r="E1265" t="n">
+        <v>566.61</v>
+      </c>
+      <c r="F1265" t="n">
+        <v>566.61</v>
+      </c>
+      <c r="G1265" t="n">
+        <v>540.0700000000001</v>
+      </c>
+      <c r="H1265" t="n">
+        <v>534.5599999999999</v>
+      </c>
+      <c r="I1265" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J1265" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1265" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 528.84 &lt;= Upper 566.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="D1266" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="E1266" t="n">
+        <v>9.029999999999999</v>
+      </c>
+      <c r="F1266" t="n">
+        <v>9.029999999999999</v>
+      </c>
+      <c r="G1266" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="H1266" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="I1266" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J1266" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1266" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7.98 &lt;= EMA21 8.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D1267" t="n">
+        <v>106.79</v>
+      </c>
+      <c r="E1267" t="n">
+        <v>109.47</v>
+      </c>
+      <c r="F1267" t="n">
+        <v>109.47</v>
+      </c>
+      <c r="G1267" t="n">
+        <v>107.14</v>
+      </c>
+      <c r="H1267" t="n">
+        <v>107.54</v>
+      </c>
+      <c r="I1267" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J1267" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1267" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 107.14 &lt;= EMA21 107.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D1268" t="n">
+        <v>893.9299999999999</v>
+      </c>
+      <c r="E1268" t="n">
+        <v>973</v>
+      </c>
+      <c r="F1268" t="n">
+        <v>973</v>
+      </c>
+      <c r="G1268" t="n">
+        <v>906.88</v>
+      </c>
+      <c r="H1268" t="n">
+        <v>921.21</v>
+      </c>
+      <c r="I1268" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J1268" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1268" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 906.88 &lt;= EMA21 921.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="D1269" t="n">
+        <v>159.83</v>
+      </c>
+      <c r="E1269" t="n">
+        <v>169.79</v>
+      </c>
+      <c r="F1269" t="n">
+        <v>169.79</v>
+      </c>
+      <c r="G1269" t="n">
+        <v>158.14</v>
+      </c>
+      <c r="H1269" t="n">
+        <v>157.97</v>
+      </c>
+      <c r="I1269" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J1269" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1269" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 159.83 &lt;= Upper 169.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D1270" t="n">
+        <v>302.51</v>
+      </c>
+      <c r="E1270" t="n">
+        <v>341.65</v>
+      </c>
+      <c r="F1270" t="n">
+        <v>341.65</v>
+      </c>
+      <c r="G1270" t="n">
+        <v>308.91</v>
+      </c>
+      <c r="H1270" t="n">
+        <v>317.38</v>
+      </c>
+      <c r="I1270" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J1270" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1270" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 308.91 &lt;= EMA21 317.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D1271" t="n">
+        <v>194.19</v>
+      </c>
+      <c r="E1271" t="n">
+        <v>219.43</v>
+      </c>
+      <c r="F1271" t="n">
+        <v>219.43</v>
+      </c>
+      <c r="G1271" t="n">
+        <v>197.45</v>
+      </c>
+      <c r="H1271" t="n">
+        <v>202.53</v>
+      </c>
+      <c r="I1271" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J1271" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1271" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 197.45 &lt;= EMA21 202.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D1272" t="n">
+        <v>60.75</v>
+      </c>
+      <c r="E1272" t="n">
+        <v>61.74</v>
+      </c>
+      <c r="F1272" t="n">
+        <v>61.74</v>
+      </c>
+      <c r="G1272" t="n">
+        <v>59.76</v>
+      </c>
+      <c r="H1272" t="n">
+        <v>58.73</v>
+      </c>
+      <c r="I1272" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J1272" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1272" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 60.75 &lt;= Upper 61.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="D1273" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="E1273" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="F1273" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="G1273" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="H1273" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="I1273" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1273" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1273" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 12.56 &lt;= Upper 12.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="D1274" t="n">
+        <v>124.95</v>
+      </c>
+      <c r="E1274" t="n">
+        <v>132.98</v>
+      </c>
+      <c r="F1274" t="n">
+        <v>132.98</v>
+      </c>
+      <c r="G1274" t="n">
+        <v>125.6</v>
+      </c>
+      <c r="H1274" t="n">
+        <v>125.52</v>
+      </c>
+      <c r="I1274" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1274" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1274" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 124.95 &lt;= Upper 132.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D1275" t="n">
+        <v>114.4</v>
+      </c>
+      <c r="E1275" t="n">
+        <v>140.7</v>
+      </c>
+      <c r="F1275" t="n">
+        <v>140.7</v>
+      </c>
+      <c r="G1275" t="n">
+        <v>118.3</v>
+      </c>
+      <c r="H1275" t="n">
+        <v>122.83</v>
+      </c>
+      <c r="I1275" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J1275" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1275" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 118.30 &lt;= EMA21 122.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D1276" t="n">
+        <v>93.34</v>
+      </c>
+      <c r="E1276" t="n">
+        <v>97.59</v>
+      </c>
+      <c r="F1276" t="n">
+        <v>97.59</v>
+      </c>
+      <c r="G1276" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="H1276" t="n">
+        <v>92.75</v>
+      </c>
+      <c r="I1276" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J1276" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1276" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 93.34 &lt;= Upper 97.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D1277" t="n">
+        <v>229.48</v>
+      </c>
+      <c r="E1277" t="n">
+        <v>240.19</v>
+      </c>
+      <c r="F1277" t="n">
+        <v>240.19</v>
+      </c>
+      <c r="G1277" t="n">
+        <v>228.37</v>
+      </c>
+      <c r="H1277" t="n">
+        <v>231.15</v>
+      </c>
+      <c r="I1277" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1277" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1277" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 228.37 &lt;= EMA21 231.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="D1278" t="n">
+        <v>126.55</v>
+      </c>
+      <c r="E1278" t="n">
+        <v>143.49</v>
+      </c>
+      <c r="F1278" t="n">
+        <v>143.49</v>
+      </c>
+      <c r="G1278" t="n">
+        <v>127.08</v>
+      </c>
+      <c r="H1278" t="n">
+        <v>132.84</v>
+      </c>
+      <c r="I1278" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J1278" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1278" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 127.08 &lt;= EMA21 132.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D1279" t="n">
+        <v>36.36</v>
+      </c>
+      <c r="E1279" t="n">
+        <v>40.71</v>
+      </c>
+      <c r="F1279" t="n">
+        <v>40.71</v>
+      </c>
+      <c r="G1279" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="H1279" t="n">
+        <v>37.99</v>
+      </c>
+      <c r="I1279" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J1279" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1279" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 36.90 &lt;= EMA21 37.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D1280" t="n">
+        <v>99.39</v>
+      </c>
+      <c r="E1280" t="n">
+        <v>130.96</v>
+      </c>
+      <c r="F1280" t="n">
+        <v>130.96</v>
+      </c>
+      <c r="G1280" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="H1280" t="n">
+        <v>107.76</v>
+      </c>
+      <c r="I1280" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1280" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1280" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 101.55 &lt;= EMA21 107.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D1281" t="n">
+        <v>96.67</v>
+      </c>
+      <c r="E1281" t="n">
+        <v>111.69</v>
+      </c>
+      <c r="F1281" t="n">
+        <v>111.69</v>
+      </c>
+      <c r="G1281" t="n">
+        <v>99.33</v>
+      </c>
+      <c r="H1281" t="n">
+        <v>101.94</v>
+      </c>
+      <c r="I1281" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1281" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1281" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 99.33 &lt;= EMA21 101.94)</t>
         </is>
       </c>
     </row>
@@ -50630,7 +54876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51502,6 +55748,68 @@
         <v>1.53</v>
       </c>
       <c r="G28" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>545.09</v>
+      </c>
+      <c r="E29" t="n">
+        <v>520.5599999999999</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="E30" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -51518,7 +55826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51599,10 +55907,10 @@
         <v>1961.07</v>
       </c>
       <c r="F2" t="n">
-        <v>673.3099999999999</v>
+        <v>682.3099999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>4.38</v>
       </c>
       <c r="H2" t="n">
         <v>654.47</v>
@@ -51611,7 +55919,7 @@
         <v>685.3099975585938</v>
       </c>
       <c r="J2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -51622,7 +55930,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -51631,28 +55939,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>330.36</v>
+        <v>60.91</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="E3" t="n">
-        <v>1982.16</v>
+        <v>1949.12</v>
       </c>
       <c r="F3" t="n">
-        <v>324.65</v>
+        <v>60.75</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.73</v>
+        <v>-0.26</v>
       </c>
       <c r="H3" t="n">
-        <v>319.51</v>
+        <v>59.62</v>
       </c>
       <c r="I3" t="n">
-        <v>334.5700073242188</v>
+        <v>62.43000030517578</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -51663,39 +55971,80 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>60.91</v>
+        <v>108.8</v>
       </c>
       <c r="D4" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>1949.12</v>
+        <v>1958.4</v>
       </c>
       <c r="F4" t="n">
-        <v>61.14</v>
+        <v>108.8</v>
       </c>
       <c r="G4" t="n">
-        <v>0.38</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>59.62</v>
+        <v>103.9</v>
       </c>
       <c r="I4" t="n">
-        <v>62.43000030517578</v>
+        <v>108.8</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>545.09</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1635.27</v>
+      </c>
+      <c r="F5" t="n">
+        <v>545.09</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>520.5599999999999</v>
+      </c>
+      <c r="I5" t="n">
+        <v>545.09</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -51712,7 +56061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52338,6 +56687,57 @@
         <v>1</v>
       </c>
       <c r="M12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>330.36</v>
+      </c>
+      <c r="E13" t="n">
+        <v>320.59</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1982.16</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-2.957</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-3.007</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-59.6</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -52354,7 +56754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53587,6 +57987,153 @@
       <c r="K25" t="inlineStr">
         <is>
           <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-18 05:03:24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CCF554123E</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>320.59</v>
+      </c>
+      <c r="G26" t="n">
+        <v>320.59</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>6</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-18 05:03:25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>F998BD0CAB</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="G27" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>18</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-18 05:03:25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>E05E9B1D02</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>545.09</v>
+      </c>
+      <c r="G28" t="n">
+        <v>545.09</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
         </is>
       </c>
     </row>
@@ -53601,7 +58148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53898,6 +58445,33 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>Qualified breakout on FFIV skipped: all slots full or insufficient cash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-18 05:03:24</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>GAP_DOWN_SLIP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Opened at 320.59 below SL of 321.74. Filled at Open.</t>
         </is>
       </c>
     </row>
@@ -53912,7 +58486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54490,6 +59064,39 @@
         <v>3</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>05:03:26</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1878.95</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7503.86</v>
+      </c>
+      <c r="E18" t="n">
+        <v>9382.809999999999</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-617.1900000000001</v>
+      </c>
+      <c r="G18" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="H18" t="n">
+        <v>12</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-19T04:47 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1281"/>
+  <dimension ref="A1:K1381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54862,6 +54862,4252 @@
       <c r="K1281" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 99.33 &lt;= EMA21 101.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D1282" t="n">
+        <v>336.13</v>
+      </c>
+      <c r="E1282" t="n">
+        <v>341.01</v>
+      </c>
+      <c r="F1282" t="n">
+        <v>341.01</v>
+      </c>
+      <c r="G1282" t="n">
+        <v>330.59</v>
+      </c>
+      <c r="H1282" t="n">
+        <v>324.65</v>
+      </c>
+      <c r="I1282" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="J1282" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1282" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 336.13 &lt;= Upper 341.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D1283" t="n">
+        <v>493.78</v>
+      </c>
+      <c r="E1283" t="n">
+        <v>512.96</v>
+      </c>
+      <c r="F1283" t="n">
+        <v>512.96</v>
+      </c>
+      <c r="G1283" t="n">
+        <v>496.13</v>
+      </c>
+      <c r="H1283" t="n">
+        <v>492.58</v>
+      </c>
+      <c r="I1283" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="J1283" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1283" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 493.78 &lt;= Upper 512.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D1284" t="n">
+        <v>222.27</v>
+      </c>
+      <c r="E1284" t="n">
+        <v>231.65</v>
+      </c>
+      <c r="F1284" t="n">
+        <v>231.65</v>
+      </c>
+      <c r="G1284" t="n">
+        <v>218.51</v>
+      </c>
+      <c r="H1284" t="n">
+        <v>218.3</v>
+      </c>
+      <c r="I1284" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J1284" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1284" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 222.27 &lt;= Upper 231.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D1285" t="n">
+        <v>349.54</v>
+      </c>
+      <c r="E1285" t="n">
+        <v>352.66</v>
+      </c>
+      <c r="F1285" t="n">
+        <v>352.66</v>
+      </c>
+      <c r="G1285" t="n">
+        <v>343.87</v>
+      </c>
+      <c r="H1285" t="n">
+        <v>343.08</v>
+      </c>
+      <c r="I1285" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="J1285" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1285" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 349.54 &lt;= Upper 352.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D1286" t="n">
+        <v>344.41</v>
+      </c>
+      <c r="E1286" t="n">
+        <v>348.44</v>
+      </c>
+      <c r="F1286" t="n">
+        <v>348.44</v>
+      </c>
+      <c r="G1286" t="n">
+        <v>340.2</v>
+      </c>
+      <c r="H1286" t="n">
+        <v>339.87</v>
+      </c>
+      <c r="I1286" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1286" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1286" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 344.41 &lt;= Upper 348.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D1287" t="n">
+        <v>253.71</v>
+      </c>
+      <c r="E1287" t="n">
+        <v>265.88</v>
+      </c>
+      <c r="F1287" t="n">
+        <v>265.88</v>
+      </c>
+      <c r="G1287" t="n">
+        <v>252.62</v>
+      </c>
+      <c r="H1287" t="n">
+        <v>255.18</v>
+      </c>
+      <c r="I1287" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="J1287" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1287" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 252.62 &lt;= EMA21 255.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D1288" t="n">
+        <v>665.75</v>
+      </c>
+      <c r="E1288" t="n">
+        <v>703.38</v>
+      </c>
+      <c r="F1288" t="n">
+        <v>703.38</v>
+      </c>
+      <c r="G1288" t="n">
+        <v>655.0599999999999</v>
+      </c>
+      <c r="H1288" t="n">
+        <v>628.27</v>
+      </c>
+      <c r="I1288" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="J1288" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1288" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 665.75 &lt;= Upper 703.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D1289" t="n">
+        <v>364.27</v>
+      </c>
+      <c r="E1289" t="n">
+        <v>375.56</v>
+      </c>
+      <c r="F1289" t="n">
+        <v>375.56</v>
+      </c>
+      <c r="G1289" t="n">
+        <v>361.95</v>
+      </c>
+      <c r="H1289" t="n">
+        <v>358.13</v>
+      </c>
+      <c r="I1289" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1289" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1289" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 364.27 &lt;= Upper 375.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D1290" t="n">
+        <v>357.61</v>
+      </c>
+      <c r="E1290" t="n">
+        <v>379.41</v>
+      </c>
+      <c r="F1290" t="n">
+        <v>379.41</v>
+      </c>
+      <c r="G1290" t="n">
+        <v>352.84</v>
+      </c>
+      <c r="H1290" t="n">
+        <v>361.54</v>
+      </c>
+      <c r="I1290" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J1290" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1290" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.84 &lt;= EMA21 361.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D1291" t="n">
+        <v>147.61</v>
+      </c>
+      <c r="E1291" t="n">
+        <v>162.04</v>
+      </c>
+      <c r="F1291" t="n">
+        <v>162.04</v>
+      </c>
+      <c r="G1291" t="n">
+        <v>148.42</v>
+      </c>
+      <c r="H1291" t="n">
+        <v>148.35</v>
+      </c>
+      <c r="I1291" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J1291" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1291" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 147.61 &lt;= Upper 162.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D1292" t="n">
+        <v>237.92</v>
+      </c>
+      <c r="E1292" t="n">
+        <v>281.86</v>
+      </c>
+      <c r="F1292" t="n">
+        <v>281.86</v>
+      </c>
+      <c r="G1292" t="n">
+        <v>246.41</v>
+      </c>
+      <c r="H1292" t="n">
+        <v>238.07</v>
+      </c>
+      <c r="I1292" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1292" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1292" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 237.92 &lt;= Upper 281.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D1293" t="n">
+        <v>248.92</v>
+      </c>
+      <c r="E1293" t="n">
+        <v>299.69</v>
+      </c>
+      <c r="F1293" t="n">
+        <v>299.69</v>
+      </c>
+      <c r="G1293" t="n">
+        <v>256.79</v>
+      </c>
+      <c r="H1293" t="n">
+        <v>261.75</v>
+      </c>
+      <c r="I1293" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J1293" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1293" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 256.79 &lt;= EMA21 261.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D1294" t="n">
+        <v>559.8200000000001</v>
+      </c>
+      <c r="E1294" t="n">
+        <v>550.12</v>
+      </c>
+      <c r="F1294" t="n">
+        <v>550.12</v>
+      </c>
+      <c r="G1294" t="n">
+        <v>518.73</v>
+      </c>
+      <c r="H1294" t="n">
+        <v>501.91</v>
+      </c>
+      <c r="I1294" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="J1294" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1294" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D1295" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="E1295" t="n">
+        <v>110.68</v>
+      </c>
+      <c r="F1295" t="n">
+        <v>110.68</v>
+      </c>
+      <c r="G1295" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="H1295" t="n">
+        <v>99.11</v>
+      </c>
+      <c r="I1295" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="J1295" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1295" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 108.60 &lt;= Upper 110.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D1296" t="n">
+        <v>1015.8</v>
+      </c>
+      <c r="E1296" t="n">
+        <v>1028.58</v>
+      </c>
+      <c r="F1296" t="n">
+        <v>1028.58</v>
+      </c>
+      <c r="G1296" t="n">
+        <v>969.52</v>
+      </c>
+      <c r="H1296" t="n">
+        <v>959.21</v>
+      </c>
+      <c r="I1296" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1296" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1296" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1015.80 &lt;= Upper 1028.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D1297" t="n">
+        <v>177.72</v>
+      </c>
+      <c r="E1297" t="n">
+        <v>191.04</v>
+      </c>
+      <c r="F1297" t="n">
+        <v>191.04</v>
+      </c>
+      <c r="G1297" t="n">
+        <v>180.13</v>
+      </c>
+      <c r="H1297" t="n">
+        <v>174.56</v>
+      </c>
+      <c r="I1297" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="J1297" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1297" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 177.72 &lt;= Upper 191.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="D1298" t="n">
+        <v>266.64</v>
+      </c>
+      <c r="E1298" t="n">
+        <v>268.88</v>
+      </c>
+      <c r="F1298" t="n">
+        <v>268.88</v>
+      </c>
+      <c r="G1298" t="n">
+        <v>262.15</v>
+      </c>
+      <c r="H1298" t="n">
+        <v>263.71</v>
+      </c>
+      <c r="I1298" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J1298" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1298" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 262.15 &lt;= EMA21 263.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D1299" t="n">
+        <v>444.57</v>
+      </c>
+      <c r="E1299" t="n">
+        <v>501.88</v>
+      </c>
+      <c r="F1299" t="n">
+        <v>501.88</v>
+      </c>
+      <c r="G1299" t="n">
+        <v>437.62</v>
+      </c>
+      <c r="H1299" t="n">
+        <v>456.75</v>
+      </c>
+      <c r="I1299" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="J1299" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1299" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 437.62 &lt;= EMA21 456.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D1300" t="n">
+        <v>288.11</v>
+      </c>
+      <c r="E1300" t="n">
+        <v>331.94</v>
+      </c>
+      <c r="F1300" t="n">
+        <v>331.94</v>
+      </c>
+      <c r="G1300" t="n">
+        <v>285.06</v>
+      </c>
+      <c r="H1300" t="n">
+        <v>295.27</v>
+      </c>
+      <c r="I1300" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J1300" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1300" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 285.06 &lt;= EMA21 295.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D1301" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="E1301" t="n">
+        <v>190.8</v>
+      </c>
+      <c r="F1301" t="n">
+        <v>190.8</v>
+      </c>
+      <c r="G1301" t="n">
+        <v>174.12</v>
+      </c>
+      <c r="H1301" t="n">
+        <v>179.25</v>
+      </c>
+      <c r="I1301" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J1301" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1301" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 174.12 &lt;= EMA21 179.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D1302" t="n">
+        <v>1679.92</v>
+      </c>
+      <c r="E1302" t="n">
+        <v>1802.6</v>
+      </c>
+      <c r="F1302" t="n">
+        <v>1802.6</v>
+      </c>
+      <c r="G1302" t="n">
+        <v>1653.88</v>
+      </c>
+      <c r="H1302" t="n">
+        <v>1683.55</v>
+      </c>
+      <c r="I1302" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1302" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1302" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1653.88 &lt;= EMA21 1683.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D1303" t="n">
+        <v>375.72</v>
+      </c>
+      <c r="E1303" t="n">
+        <v>378.85</v>
+      </c>
+      <c r="F1303" t="n">
+        <v>378.85</v>
+      </c>
+      <c r="G1303" t="n">
+        <v>366</v>
+      </c>
+      <c r="H1303" t="n">
+        <v>367.01</v>
+      </c>
+      <c r="I1303" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="J1303" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1303" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 366.00 &lt;= EMA21 367.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D1304" t="n">
+        <v>244.25</v>
+      </c>
+      <c r="E1304" t="n">
+        <v>252.35</v>
+      </c>
+      <c r="F1304" t="n">
+        <v>252.35</v>
+      </c>
+      <c r="G1304" t="n">
+        <v>231.64</v>
+      </c>
+      <c r="H1304" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="I1304" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J1304" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1304" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 244.25 &lt;= Upper 252.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="D1305" t="n">
+        <v>227.99</v>
+      </c>
+      <c r="E1305" t="n">
+        <v>231.59</v>
+      </c>
+      <c r="F1305" t="n">
+        <v>231.59</v>
+      </c>
+      <c r="G1305" t="n">
+        <v>225.72</v>
+      </c>
+      <c r="H1305" t="n">
+        <v>227.3</v>
+      </c>
+      <c r="I1305" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J1305" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1305" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 225.72 &lt;= EMA21 227.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D1306" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="E1306" t="n">
+        <v>76.77</v>
+      </c>
+      <c r="F1306" t="n">
+        <v>76.77</v>
+      </c>
+      <c r="G1306" t="n">
+        <v>70.77</v>
+      </c>
+      <c r="H1306" t="n">
+        <v>73.16</v>
+      </c>
+      <c r="I1306" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="J1306" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1306" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 70.77 &lt;= EMA21 73.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D1307" t="n">
+        <v>1217.8</v>
+      </c>
+      <c r="E1307" t="n">
+        <v>1341.08</v>
+      </c>
+      <c r="F1307" t="n">
+        <v>1341.08</v>
+      </c>
+      <c r="G1307" t="n">
+        <v>1190.84</v>
+      </c>
+      <c r="H1307" t="n">
+        <v>1229.06</v>
+      </c>
+      <c r="I1307" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="J1307" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1307" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1190.84 &lt;= EMA21 1229.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D1308" t="n">
+        <v>88.76000000000001</v>
+      </c>
+      <c r="E1308" t="n">
+        <v>94.11</v>
+      </c>
+      <c r="F1308" t="n">
+        <v>94.11</v>
+      </c>
+      <c r="G1308" t="n">
+        <v>84.31999999999999</v>
+      </c>
+      <c r="H1308" t="n">
+        <v>78.09</v>
+      </c>
+      <c r="I1308" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="J1308" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1308" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 88.76 &lt;= Upper 94.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D1309" t="n">
+        <v>117.18</v>
+      </c>
+      <c r="E1309" t="n">
+        <v>122.31</v>
+      </c>
+      <c r="F1309" t="n">
+        <v>122.31</v>
+      </c>
+      <c r="G1309" t="n">
+        <v>112.75</v>
+      </c>
+      <c r="H1309" t="n">
+        <v>106.53</v>
+      </c>
+      <c r="I1309" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="J1309" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1309" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 117.18 &lt;= Upper 122.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D1310" t="n">
+        <v>371.47</v>
+      </c>
+      <c r="E1310" t="n">
+        <v>391.05</v>
+      </c>
+      <c r="F1310" t="n">
+        <v>391.05</v>
+      </c>
+      <c r="G1310" t="n">
+        <v>355.94</v>
+      </c>
+      <c r="H1310" t="n">
+        <v>360.58</v>
+      </c>
+      <c r="I1310" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J1310" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1310" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 355.94 &lt;= EMA21 360.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>ENTG</t>
+        </is>
+      </c>
+      <c r="D1311" t="n">
+        <v>142.25</v>
+      </c>
+      <c r="E1311" t="n">
+        <v>147.63</v>
+      </c>
+      <c r="F1311" t="n">
+        <v>147.63</v>
+      </c>
+      <c r="G1311" t="n">
+        <v>135.93</v>
+      </c>
+      <c r="H1311" t="n">
+        <v>137.56</v>
+      </c>
+      <c r="I1311" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J1311" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1311" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.93 &lt;= EMA21 137.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+      <c r="D1312" t="n">
+        <v>73.27</v>
+      </c>
+      <c r="E1312" t="n">
+        <v>76.04000000000001</v>
+      </c>
+      <c r="F1312" t="n">
+        <v>76.04000000000001</v>
+      </c>
+      <c r="G1312" t="n">
+        <v>72.11</v>
+      </c>
+      <c r="H1312" t="n">
+        <v>73.42</v>
+      </c>
+      <c r="I1312" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="J1312" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1312" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 72.11 &lt;= EMA21 73.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D1313" t="n">
+        <v>39.09</v>
+      </c>
+      <c r="E1313" t="n">
+        <v>40.84</v>
+      </c>
+      <c r="F1313" t="n">
+        <v>40.84</v>
+      </c>
+      <c r="G1313" t="n">
+        <v>38.28</v>
+      </c>
+      <c r="H1313" t="n">
+        <v>37.43</v>
+      </c>
+      <c r="I1313" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J1313" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1313" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 39.09 &lt;= Upper 40.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D1314" t="n">
+        <v>568.0599999999999</v>
+      </c>
+      <c r="E1314" t="n">
+        <v>605.08</v>
+      </c>
+      <c r="F1314" t="n">
+        <v>605.08</v>
+      </c>
+      <c r="G1314" t="n">
+        <v>547.9299999999999</v>
+      </c>
+      <c r="H1314" t="n">
+        <v>515.4400000000001</v>
+      </c>
+      <c r="I1314" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J1314" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1314" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 568.06 &lt;= Upper 605.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D1315" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="E1315" t="n">
+        <v>35.84</v>
+      </c>
+      <c r="F1315" t="n">
+        <v>35.84</v>
+      </c>
+      <c r="G1315" t="n">
+        <v>33.44</v>
+      </c>
+      <c r="H1315" t="n">
+        <v>32</v>
+      </c>
+      <c r="I1315" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="J1315" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1315" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 34.40 &lt;= Upper 35.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="D1316" t="n">
+        <v>441.36</v>
+      </c>
+      <c r="E1316" t="n">
+        <v>487.44</v>
+      </c>
+      <c r="F1316" t="n">
+        <v>487.44</v>
+      </c>
+      <c r="G1316" t="n">
+        <v>437.63</v>
+      </c>
+      <c r="H1316" t="n">
+        <v>451.42</v>
+      </c>
+      <c r="I1316" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="J1316" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1316" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 437.63 &lt;= EMA21 451.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D1317" t="n">
+        <v>858.79</v>
+      </c>
+      <c r="E1317" t="n">
+        <v>897.4299999999999</v>
+      </c>
+      <c r="F1317" t="n">
+        <v>897.4299999999999</v>
+      </c>
+      <c r="G1317" t="n">
+        <v>824.01</v>
+      </c>
+      <c r="H1317" t="n">
+        <v>833.55</v>
+      </c>
+      <c r="I1317" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="J1317" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1317" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 824.01 &lt;= EMA21 833.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="D1318" t="n">
+        <v>199.39</v>
+      </c>
+      <c r="E1318" t="n">
+        <v>203.62</v>
+      </c>
+      <c r="F1318" t="n">
+        <v>203.62</v>
+      </c>
+      <c r="G1318" t="n">
+        <v>195.67</v>
+      </c>
+      <c r="H1318" t="n">
+        <v>193.62</v>
+      </c>
+      <c r="I1318" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="J1318" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1318" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 199.39 &lt;= Upper 203.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D1319" t="n">
+        <v>109.51</v>
+      </c>
+      <c r="E1319" t="n">
+        <v>112.65</v>
+      </c>
+      <c r="F1319" t="n">
+        <v>112.65</v>
+      </c>
+      <c r="G1319" t="n">
+        <v>109.64</v>
+      </c>
+      <c r="H1319" t="n">
+        <v>110.56</v>
+      </c>
+      <c r="I1319" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J1319" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1319" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 109.64 &lt;= EMA21 110.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="D1320" t="n">
+        <v>181.29</v>
+      </c>
+      <c r="E1320" t="n">
+        <v>196.89</v>
+      </c>
+      <c r="F1320" t="n">
+        <v>196.89</v>
+      </c>
+      <c r="G1320" t="n">
+        <v>186.67</v>
+      </c>
+      <c r="H1320" t="n">
+        <v>184.04</v>
+      </c>
+      <c r="I1320" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="J1320" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1320" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 181.29 &lt;= Upper 196.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="D1321" t="n">
+        <v>229.55</v>
+      </c>
+      <c r="E1321" t="n">
+        <v>247.21</v>
+      </c>
+      <c r="F1321" t="n">
+        <v>247.21</v>
+      </c>
+      <c r="G1321" t="n">
+        <v>237.64</v>
+      </c>
+      <c r="H1321" t="n">
+        <v>236.73</v>
+      </c>
+      <c r="I1321" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="J1321" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1321" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 229.55 &lt;= Upper 247.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D1322" t="n">
+        <v>135.47</v>
+      </c>
+      <c r="E1322" t="n">
+        <v>150.05</v>
+      </c>
+      <c r="F1322" t="n">
+        <v>150.05</v>
+      </c>
+      <c r="G1322" t="n">
+        <v>137.55</v>
+      </c>
+      <c r="H1322" t="n">
+        <v>134.67</v>
+      </c>
+      <c r="I1322" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J1322" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1322" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 135.47 &lt;= Upper 150.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D1323" t="n">
+        <v>303.19</v>
+      </c>
+      <c r="E1323" t="n">
+        <v>376.84</v>
+      </c>
+      <c r="F1323" t="n">
+        <v>376.84</v>
+      </c>
+      <c r="G1323" t="n">
+        <v>320.76</v>
+      </c>
+      <c r="H1323" t="n">
+        <v>328.67</v>
+      </c>
+      <c r="I1323" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J1323" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1323" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 320.76 &lt;= EMA21 328.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D1324" t="n">
+        <v>363.58</v>
+      </c>
+      <c r="E1324" t="n">
+        <v>393.4</v>
+      </c>
+      <c r="F1324" t="n">
+        <v>393.4</v>
+      </c>
+      <c r="G1324" t="n">
+        <v>361.46</v>
+      </c>
+      <c r="H1324" t="n">
+        <v>357.13</v>
+      </c>
+      <c r="I1324" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J1324" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1324" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 363.58 &lt;= Upper 393.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D1325" t="n">
+        <v>237.65</v>
+      </c>
+      <c r="E1325" t="n">
+        <v>253.49</v>
+      </c>
+      <c r="F1325" t="n">
+        <v>253.49</v>
+      </c>
+      <c r="G1325" t="n">
+        <v>230.5</v>
+      </c>
+      <c r="H1325" t="n">
+        <v>220.47</v>
+      </c>
+      <c r="I1325" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J1325" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1325" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 237.65 &lt;= Upper 253.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D1326" t="n">
+        <v>332.43</v>
+      </c>
+      <c r="E1326" t="n">
+        <v>349.62</v>
+      </c>
+      <c r="F1326" t="n">
+        <v>349.62</v>
+      </c>
+      <c r="G1326" t="n">
+        <v>331.58</v>
+      </c>
+      <c r="H1326" t="n">
+        <v>327.68</v>
+      </c>
+      <c r="I1326" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1326" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1326" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 332.43 &lt;= Upper 349.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D1327" t="n">
+        <v>177.64</v>
+      </c>
+      <c r="E1327" t="n">
+        <v>188.23</v>
+      </c>
+      <c r="F1327" t="n">
+        <v>188.23</v>
+      </c>
+      <c r="G1327" t="n">
+        <v>174.26</v>
+      </c>
+      <c r="H1327" t="n">
+        <v>172.37</v>
+      </c>
+      <c r="I1327" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J1327" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1327" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 177.64 &lt;= Upper 188.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D1328" t="n">
+        <v>229.92</v>
+      </c>
+      <c r="E1328" t="n">
+        <v>245.06</v>
+      </c>
+      <c r="F1328" t="n">
+        <v>245.06</v>
+      </c>
+      <c r="G1328" t="n">
+        <v>228.33</v>
+      </c>
+      <c r="H1328" t="n">
+        <v>229.96</v>
+      </c>
+      <c r="I1328" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J1328" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1328" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 228.33 &lt;= EMA21 229.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D1329" t="n">
+        <v>197.31</v>
+      </c>
+      <c r="E1329" t="n">
+        <v>202.73</v>
+      </c>
+      <c r="F1329" t="n">
+        <v>202.73</v>
+      </c>
+      <c r="G1329" t="n">
+        <v>186.63</v>
+      </c>
+      <c r="H1329" t="n">
+        <v>180.12</v>
+      </c>
+      <c r="I1329" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J1329" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1329" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 197.31 &lt;= Upper 202.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D1330" t="n">
+        <v>323.6</v>
+      </c>
+      <c r="E1330" t="n">
+        <v>340.95</v>
+      </c>
+      <c r="F1330" t="n">
+        <v>340.95</v>
+      </c>
+      <c r="G1330" t="n">
+        <v>317.91</v>
+      </c>
+      <c r="H1330" t="n">
+        <v>306.82</v>
+      </c>
+      <c r="I1330" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J1330" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1330" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 323.60 &lt;= Upper 340.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="D1331" t="n">
+        <v>383.56</v>
+      </c>
+      <c r="E1331" t="n">
+        <v>456.72</v>
+      </c>
+      <c r="F1331" t="n">
+        <v>456.72</v>
+      </c>
+      <c r="G1331" t="n">
+        <v>382.45</v>
+      </c>
+      <c r="H1331" t="n">
+        <v>388.74</v>
+      </c>
+      <c r="I1331" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J1331" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1331" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 382.45 &lt;= EMA21 388.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D1332" t="n">
+        <v>169.84</v>
+      </c>
+      <c r="E1332" t="n">
+        <v>177.48</v>
+      </c>
+      <c r="F1332" t="n">
+        <v>177.48</v>
+      </c>
+      <c r="G1332" t="n">
+        <v>166.96</v>
+      </c>
+      <c r="H1332" t="n">
+        <v>163.4</v>
+      </c>
+      <c r="I1332" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="J1332" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1332" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 169.84 &lt;= Upper 177.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D1333" t="n">
+        <v>192.02</v>
+      </c>
+      <c r="E1333" t="n">
+        <v>202.12</v>
+      </c>
+      <c r="F1333" t="n">
+        <v>202.12</v>
+      </c>
+      <c r="G1333" t="n">
+        <v>188.16</v>
+      </c>
+      <c r="H1333" t="n">
+        <v>179.12</v>
+      </c>
+      <c r="I1333" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="J1333" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1333" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 192.02 &lt;= Upper 202.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>WDAY</t>
+        </is>
+      </c>
+      <c r="D1334" t="n">
+        <v>193.87</v>
+      </c>
+      <c r="E1334" t="n">
+        <v>207.36</v>
+      </c>
+      <c r="F1334" t="n">
+        <v>207.36</v>
+      </c>
+      <c r="G1334" t="n">
+        <v>192.7</v>
+      </c>
+      <c r="H1334" t="n">
+        <v>190.88</v>
+      </c>
+      <c r="I1334" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="J1334" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1334" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 193.87 &lt;= Upper 207.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="D1335" t="n">
+        <v>216.12</v>
+      </c>
+      <c r="E1335" t="n">
+        <v>266.44</v>
+      </c>
+      <c r="F1335" t="n">
+        <v>266.44</v>
+      </c>
+      <c r="G1335" t="n">
+        <v>233.13</v>
+      </c>
+      <c r="H1335" t="n">
+        <v>235.87</v>
+      </c>
+      <c r="I1335" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="J1335" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1335" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 233.13 &lt;= EMA21 235.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="D1336" t="n">
+        <v>260.21</v>
+      </c>
+      <c r="E1336" t="n">
+        <v>291.78</v>
+      </c>
+      <c r="F1336" t="n">
+        <v>291.78</v>
+      </c>
+      <c r="G1336" t="n">
+        <v>264.51</v>
+      </c>
+      <c r="H1336" t="n">
+        <v>260.21</v>
+      </c>
+      <c r="I1336" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="J1336" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1336" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 260.21 &lt;= Upper 291.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D1337" t="n">
+        <v>88.77</v>
+      </c>
+      <c r="E1337" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="F1337" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="G1337" t="n">
+        <v>93.45</v>
+      </c>
+      <c r="H1337" t="n">
+        <v>96.05</v>
+      </c>
+      <c r="I1337" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J1337" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1337" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 93.45 &lt;= EMA21 96.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D1338" t="n">
+        <v>182.37</v>
+      </c>
+      <c r="E1338" t="n">
+        <v>204.84</v>
+      </c>
+      <c r="F1338" t="n">
+        <v>204.84</v>
+      </c>
+      <c r="G1338" t="n">
+        <v>180.25</v>
+      </c>
+      <c r="H1338" t="n">
+        <v>169.67</v>
+      </c>
+      <c r="I1338" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J1338" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1338" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 182.37 &lt;= Upper 204.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="D1339" t="n">
+        <v>308.06</v>
+      </c>
+      <c r="E1339" t="n">
+        <v>333.49</v>
+      </c>
+      <c r="F1339" t="n">
+        <v>333.49</v>
+      </c>
+      <c r="G1339" t="n">
+        <v>319.5</v>
+      </c>
+      <c r="H1339" t="n">
+        <v>323.68</v>
+      </c>
+      <c r="I1339" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="J1339" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1339" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 319.50 &lt;= EMA21 323.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="D1340" t="n">
+        <v>447.76</v>
+      </c>
+      <c r="E1340" t="n">
+        <v>652.74</v>
+      </c>
+      <c r="F1340" t="n">
+        <v>652.74</v>
+      </c>
+      <c r="G1340" t="n">
+        <v>475.76</v>
+      </c>
+      <c r="H1340" t="n">
+        <v>511.72</v>
+      </c>
+      <c r="I1340" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J1340" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1340" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 475.76 &lt;= EMA21 511.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="D1341" t="n">
+        <v>282.9</v>
+      </c>
+      <c r="E1341" t="n">
+        <v>352.76</v>
+      </c>
+      <c r="F1341" t="n">
+        <v>352.76</v>
+      </c>
+      <c r="G1341" t="n">
+        <v>285.9</v>
+      </c>
+      <c r="H1341" t="n">
+        <v>299.47</v>
+      </c>
+      <c r="I1341" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J1341" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1341" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 285.90 &lt;= EMA21 299.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D1342" t="n">
+        <v>384.97</v>
+      </c>
+      <c r="E1342" t="n">
+        <v>451.49</v>
+      </c>
+      <c r="F1342" t="n">
+        <v>451.49</v>
+      </c>
+      <c r="G1342" t="n">
+        <v>387.59</v>
+      </c>
+      <c r="H1342" t="n">
+        <v>397.06</v>
+      </c>
+      <c r="I1342" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="J1342" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1342" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 387.59 &lt;= EMA21 397.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D1343" t="n">
+        <v>216.95</v>
+      </c>
+      <c r="E1343" t="n">
+        <v>275.33</v>
+      </c>
+      <c r="F1343" t="n">
+        <v>275.33</v>
+      </c>
+      <c r="G1343" t="n">
+        <v>221.94</v>
+      </c>
+      <c r="H1343" t="n">
+        <v>229.33</v>
+      </c>
+      <c r="I1343" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="J1343" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1343" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 221.94 &lt;= EMA21 229.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="J1344" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1344" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D1345" t="n">
+        <v>135.89</v>
+      </c>
+      <c r="E1345" t="n">
+        <v>165.28</v>
+      </c>
+      <c r="F1345" t="n">
+        <v>165.28</v>
+      </c>
+      <c r="G1345" t="n">
+        <v>135.6</v>
+      </c>
+      <c r="H1345" t="n">
+        <v>139.47</v>
+      </c>
+      <c r="I1345" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="J1345" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1345" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.60 &lt;= EMA21 139.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>TYL</t>
+        </is>
+      </c>
+      <c r="D1346" t="n">
+        <v>337.5</v>
+      </c>
+      <c r="E1346" t="n">
+        <v>385.59</v>
+      </c>
+      <c r="F1346" t="n">
+        <v>385.59</v>
+      </c>
+      <c r="G1346" t="n">
+        <v>347.03</v>
+      </c>
+      <c r="H1346" t="n">
+        <v>347.65</v>
+      </c>
+      <c r="I1346" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="J1346" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1346" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 347.03 &lt;= EMA21 347.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="D1347" t="n">
+        <v>143.73</v>
+      </c>
+      <c r="E1347" t="n">
+        <v>161.9</v>
+      </c>
+      <c r="F1347" t="n">
+        <v>161.9</v>
+      </c>
+      <c r="G1347" t="n">
+        <v>146.45</v>
+      </c>
+      <c r="H1347" t="n">
+        <v>147.35</v>
+      </c>
+      <c r="I1347" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J1347" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1347" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 146.45 &lt;= EMA21 147.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1348" t="n">
+        <v>185.78</v>
+      </c>
+      <c r="E1348" t="n">
+        <v>208.8</v>
+      </c>
+      <c r="F1348" t="n">
+        <v>208.8</v>
+      </c>
+      <c r="G1348" t="n">
+        <v>187.24</v>
+      </c>
+      <c r="H1348" t="n">
+        <v>185.7</v>
+      </c>
+      <c r="I1348" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="J1348" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1348" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 185.78 &lt;= Upper 208.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D1349" t="n">
+        <v>59.87</v>
+      </c>
+      <c r="E1349" t="n">
+        <v>66.05</v>
+      </c>
+      <c r="F1349" t="n">
+        <v>66.05</v>
+      </c>
+      <c r="G1349" t="n">
+        <v>61.42</v>
+      </c>
+      <c r="H1349" t="n">
+        <v>60.81</v>
+      </c>
+      <c r="I1349" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="J1349" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1349" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 59.87 &lt;= Upper 66.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1350" t="n">
+        <v>10.82</v>
+      </c>
+      <c r="E1350" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="F1350" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="G1350" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="H1350" t="n">
+        <v>11.46</v>
+      </c>
+      <c r="I1350" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1350" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1350" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11.19 &lt;= EMA21 11.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D1351" t="n">
+        <v>114</v>
+      </c>
+      <c r="E1351" t="n">
+        <v>123.46</v>
+      </c>
+      <c r="F1351" t="n">
+        <v>123.46</v>
+      </c>
+      <c r="G1351" t="n">
+        <v>117.17</v>
+      </c>
+      <c r="H1351" t="n">
+        <v>114.33</v>
+      </c>
+      <c r="I1351" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J1351" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1351" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 114.00 &lt;= Upper 123.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>GEN</t>
+        </is>
+      </c>
+      <c r="D1352" t="n">
+        <v>29.01</v>
+      </c>
+      <c r="E1352" t="n">
+        <v>31.78</v>
+      </c>
+      <c r="F1352" t="n">
+        <v>31.78</v>
+      </c>
+      <c r="G1352" t="n">
+        <v>30.21</v>
+      </c>
+      <c r="H1352" t="n">
+        <v>29.91</v>
+      </c>
+      <c r="I1352" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="J1352" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1352" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 29.01 &lt;= Upper 31.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D1353" t="n">
+        <v>146.19</v>
+      </c>
+      <c r="E1353" t="n">
+        <v>158.97</v>
+      </c>
+      <c r="F1353" t="n">
+        <v>158.97</v>
+      </c>
+      <c r="G1353" t="n">
+        <v>148.76</v>
+      </c>
+      <c r="H1353" t="n">
+        <v>146.66</v>
+      </c>
+      <c r="I1353" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="J1353" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1353" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 146.19 &lt;= Upper 158.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D1354" t="n">
+        <v>432.03</v>
+      </c>
+      <c r="E1354" t="n">
+        <v>436.74</v>
+      </c>
+      <c r="F1354" t="n">
+        <v>436.74</v>
+      </c>
+      <c r="G1354" t="n">
+        <v>418.81</v>
+      </c>
+      <c r="H1354" t="n">
+        <v>409.24</v>
+      </c>
+      <c r="I1354" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J1354" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1354" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 432.03 &lt;= Upper 436.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>JNPR</t>
+        </is>
+      </c>
+      <c r="J1355" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1355" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="D1356" t="n">
+        <v>104.52</v>
+      </c>
+      <c r="E1356" t="n">
+        <v>110.92</v>
+      </c>
+      <c r="F1356" t="n">
+        <v>110.92</v>
+      </c>
+      <c r="G1356" t="n">
+        <v>106.09</v>
+      </c>
+      <c r="H1356" t="n">
+        <v>108.17</v>
+      </c>
+      <c r="I1356" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J1356" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1356" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.09 &lt;= EMA21 108.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="J1357" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1357" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="D1358" t="n">
+        <v>205.45</v>
+      </c>
+      <c r="E1358" t="n">
+        <v>240.96</v>
+      </c>
+      <c r="F1358" t="n">
+        <v>240.96</v>
+      </c>
+      <c r="G1358" t="n">
+        <v>213.23</v>
+      </c>
+      <c r="H1358" t="n">
+        <v>220.1</v>
+      </c>
+      <c r="I1358" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="J1358" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1358" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 213.23 &lt;= EMA21 220.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D1359" t="n">
+        <v>47.82</v>
+      </c>
+      <c r="E1359" t="n">
+        <v>51.59</v>
+      </c>
+      <c r="F1359" t="n">
+        <v>51.59</v>
+      </c>
+      <c r="G1359" t="n">
+        <v>46.75</v>
+      </c>
+      <c r="H1359" t="n">
+        <v>44.45</v>
+      </c>
+      <c r="I1359" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J1359" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1359" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 47.82 &lt;= Upper 51.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D1360" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="E1360" t="n">
+        <v>46.28</v>
+      </c>
+      <c r="F1360" t="n">
+        <v>46.28</v>
+      </c>
+      <c r="G1360" t="n">
+        <v>42.34</v>
+      </c>
+      <c r="H1360" t="n">
+        <v>42.27</v>
+      </c>
+      <c r="I1360" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J1360" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1360" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 41.40 &lt;= Upper 46.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D1361" t="n">
+        <v>71.79000000000001</v>
+      </c>
+      <c r="E1361" t="n">
+        <v>84.75</v>
+      </c>
+      <c r="F1361" t="n">
+        <v>84.75</v>
+      </c>
+      <c r="G1361" t="n">
+        <v>76.39</v>
+      </c>
+      <c r="H1361" t="n">
+        <v>77.43000000000001</v>
+      </c>
+      <c r="I1361" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="J1361" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1361" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 76.39 &lt;= EMA21 77.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D1362" t="n">
+        <v>102.67</v>
+      </c>
+      <c r="E1362" t="n">
+        <v>111.16</v>
+      </c>
+      <c r="F1362" t="n">
+        <v>111.16</v>
+      </c>
+      <c r="G1362" t="n">
+        <v>105.67</v>
+      </c>
+      <c r="H1362" t="n">
+        <v>105.74</v>
+      </c>
+      <c r="I1362" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="J1362" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1362" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 105.67 &lt;= EMA21 105.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="D1363" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="E1363" t="n">
+        <v>29</v>
+      </c>
+      <c r="F1363" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1363" t="n">
+        <v>28.09</v>
+      </c>
+      <c r="H1363" t="n">
+        <v>28.06</v>
+      </c>
+      <c r="I1363" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J1363" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1363" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 27.80 &lt;= Upper 29.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="D1364" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E1364" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F1364" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="G1364" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H1364" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="I1364" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J1364" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1364" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 0.99 &lt;= EMA21 1.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D1365" t="n">
+        <v>509.45</v>
+      </c>
+      <c r="E1365" t="n">
+        <v>568.9299999999999</v>
+      </c>
+      <c r="F1365" t="n">
+        <v>568.9299999999999</v>
+      </c>
+      <c r="G1365" t="n">
+        <v>533.95</v>
+      </c>
+      <c r="H1365" t="n">
+        <v>532.28</v>
+      </c>
+      <c r="I1365" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J1365" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1365" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 509.45 &lt;= Upper 568.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="D1366" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="E1366" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="F1366" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="G1366" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="H1366" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="I1366" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="J1366" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1366" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7.94 &lt;= EMA21 8.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D1367" t="n">
+        <v>106.73</v>
+      </c>
+      <c r="E1367" t="n">
+        <v>109.47</v>
+      </c>
+      <c r="F1367" t="n">
+        <v>109.47</v>
+      </c>
+      <c r="G1367" t="n">
+        <v>107.06</v>
+      </c>
+      <c r="H1367" t="n">
+        <v>107.46</v>
+      </c>
+      <c r="I1367" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J1367" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1367" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 107.06 &lt;= EMA21 107.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D1368" t="n">
+        <v>895.3099999999999</v>
+      </c>
+      <c r="E1368" t="n">
+        <v>972.98</v>
+      </c>
+      <c r="F1368" t="n">
+        <v>972.98</v>
+      </c>
+      <c r="G1368" t="n">
+        <v>904.5700000000001</v>
+      </c>
+      <c r="H1368" t="n">
+        <v>918.86</v>
+      </c>
+      <c r="I1368" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="J1368" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1368" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 904.57 &lt;= EMA21 918.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="D1369" t="n">
+        <v>158.19</v>
+      </c>
+      <c r="E1369" t="n">
+        <v>169.8</v>
+      </c>
+      <c r="F1369" t="n">
+        <v>169.8</v>
+      </c>
+      <c r="G1369" t="n">
+        <v>158.15</v>
+      </c>
+      <c r="H1369" t="n">
+        <v>157.99</v>
+      </c>
+      <c r="I1369" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="J1369" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1369" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 158.19 &lt;= Upper 169.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D1370" t="n">
+        <v>299.98</v>
+      </c>
+      <c r="E1370" t="n">
+        <v>340.69</v>
+      </c>
+      <c r="F1370" t="n">
+        <v>340.69</v>
+      </c>
+      <c r="G1370" t="n">
+        <v>307.12</v>
+      </c>
+      <c r="H1370" t="n">
+        <v>315.8</v>
+      </c>
+      <c r="I1370" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="J1370" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1370" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 307.12 &lt;= EMA21 315.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D1371" t="n">
+        <v>192.49</v>
+      </c>
+      <c r="E1371" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="F1371" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="G1371" t="n">
+        <v>196.45</v>
+      </c>
+      <c r="H1371" t="n">
+        <v>201.62</v>
+      </c>
+      <c r="I1371" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J1371" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1371" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 196.45 &lt;= EMA21 201.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D1372" t="n">
+        <v>60</v>
+      </c>
+      <c r="E1372" t="n">
+        <v>61.82</v>
+      </c>
+      <c r="F1372" t="n">
+        <v>61.82</v>
+      </c>
+      <c r="G1372" t="n">
+        <v>59.81</v>
+      </c>
+      <c r="H1372" t="n">
+        <v>58.85</v>
+      </c>
+      <c r="I1372" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="J1372" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1372" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 60.00 &lt;= Upper 61.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="D1373" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="E1373" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="F1373" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="G1373" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="H1373" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="I1373" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="J1373" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1373" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 12.35 &lt;= Upper 12.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="D1374" t="n">
+        <v>122.41</v>
+      </c>
+      <c r="E1374" t="n">
+        <v>132.83</v>
+      </c>
+      <c r="F1374" t="n">
+        <v>132.83</v>
+      </c>
+      <c r="G1374" t="n">
+        <v>124.96</v>
+      </c>
+      <c r="H1374" t="n">
+        <v>125.23</v>
+      </c>
+      <c r="I1374" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="J1374" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1374" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 124.96 &lt;= EMA21 125.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D1375" t="n">
+        <v>111.96</v>
+      </c>
+      <c r="E1375" t="n">
+        <v>140.94</v>
+      </c>
+      <c r="F1375" t="n">
+        <v>140.94</v>
+      </c>
+      <c r="G1375" t="n">
+        <v>117.04</v>
+      </c>
+      <c r="H1375" t="n">
+        <v>121.84</v>
+      </c>
+      <c r="I1375" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="J1375" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1375" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 117.04 &lt;= EMA21 121.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D1376" t="n">
+        <v>92.03</v>
+      </c>
+      <c r="E1376" t="n">
+        <v>97.59999999999999</v>
+      </c>
+      <c r="F1376" t="n">
+        <v>97.59999999999999</v>
+      </c>
+      <c r="G1376" t="n">
+        <v>92.65000000000001</v>
+      </c>
+      <c r="H1376" t="n">
+        <v>92.69</v>
+      </c>
+      <c r="I1376" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1376" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1376" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 92.65 &lt;= EMA21 92.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D1377" t="n">
+        <v>226.61</v>
+      </c>
+      <c r="E1377" t="n">
+        <v>240.22</v>
+      </c>
+      <c r="F1377" t="n">
+        <v>240.22</v>
+      </c>
+      <c r="G1377" t="n">
+        <v>228.02</v>
+      </c>
+      <c r="H1377" t="n">
+        <v>230.74</v>
+      </c>
+      <c r="I1377" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="J1377" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1377" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 228.02 &lt;= EMA21 230.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="D1378" t="n">
+        <v>127.24</v>
+      </c>
+      <c r="E1378" t="n">
+        <v>142.21</v>
+      </c>
+      <c r="F1378" t="n">
+        <v>142.21</v>
+      </c>
+      <c r="G1378" t="n">
+        <v>127.12</v>
+      </c>
+      <c r="H1378" t="n">
+        <v>132.33</v>
+      </c>
+      <c r="I1378" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J1378" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1378" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 127.12 &lt;= EMA21 132.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D1379" t="n">
+        <v>35.51</v>
+      </c>
+      <c r="E1379" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="F1379" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G1379" t="n">
+        <v>36.62</v>
+      </c>
+      <c r="H1379" t="n">
+        <v>37.76</v>
+      </c>
+      <c r="I1379" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J1379" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1379" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 36.62 &lt;= EMA21 37.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D1380" t="n">
+        <v>98.06</v>
+      </c>
+      <c r="E1380" t="n">
+        <v>130.58</v>
+      </c>
+      <c r="F1380" t="n">
+        <v>130.58</v>
+      </c>
+      <c r="G1380" t="n">
+        <v>100.85</v>
+      </c>
+      <c r="H1380" t="n">
+        <v>106.88</v>
+      </c>
+      <c r="I1380" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1380" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1380" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 100.85 &lt;= EMA21 106.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D1381" t="n">
+        <v>95.83</v>
+      </c>
+      <c r="E1381" t="n">
+        <v>111.92</v>
+      </c>
+      <c r="F1381" t="n">
+        <v>111.92</v>
+      </c>
+      <c r="G1381" t="n">
+        <v>98.63</v>
+      </c>
+      <c r="H1381" t="n">
+        <v>101.39</v>
+      </c>
+      <c r="I1381" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="J1381" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1381" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 98.63 &lt;= EMA21 101.39)</t>
         </is>
       </c>
     </row>
@@ -54876,7 +59122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55810,6 +60056,37 @@
         <v>1.58</v>
       </c>
       <c r="G30" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>559.8200000000001</v>
+      </c>
+      <c r="E31" t="n">
+        <v>534.63</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="G31" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -55907,19 +60184,19 @@
         <v>1961.07</v>
       </c>
       <c r="F2" t="n">
-        <v>682.3099999999999</v>
+        <v>665.75</v>
       </c>
       <c r="G2" t="n">
-        <v>4.38</v>
+        <v>1.84</v>
       </c>
       <c r="H2" t="n">
-        <v>654.47</v>
+        <v>659.09</v>
       </c>
       <c r="I2" t="n">
-        <v>685.3099975585938</v>
+        <v>690.1500244140625</v>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -55948,10 +60225,10 @@
         <v>1949.12</v>
       </c>
       <c r="F3" t="n">
-        <v>60.75</v>
+        <v>60</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.26</v>
+        <v>-1.49</v>
       </c>
       <c r="H3" t="n">
         <v>59.62</v>
@@ -55960,7 +60237,7 @@
         <v>62.43000030517578</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -58486,7 +62763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59097,6 +63374,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>04:47:14</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1878.95</v>
+      </c>
+      <c r="D19" t="n">
+        <v>7503.86</v>
+      </c>
+      <c r="E19" t="n">
+        <v>9382.809999999999</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-617.1900000000001</v>
+      </c>
+      <c r="G19" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="H19" t="n">
+        <v>12</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>